<commit_message>
String Node in Java fixed
</commit_message>
<xml_diff>
--- a/files/Kompetenzraster.xlsx
+++ b/files/Kompetenzraster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcsauer/GitHub/hefl/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB50F974-8CB0-45A5-B96E-574579D5AE5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A2E42F9-24C8-4946-9F73-FF746C9023AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25725" yWindow="90" windowWidth="25890" windowHeight="20805" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19640" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OFP" sheetId="1" r:id="rId1"/>
@@ -2049,7 +2049,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2661,9 +2661,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2701,7 +2701,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2807,7 +2807,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2949,7 +2949,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2958,25 +2958,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I245"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="4" width="7.140625" customWidth="1"/>
+    <col min="1" max="2" width="35.6640625" customWidth="1"/>
+    <col min="3" max="4" width="7.1640625" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
-    <col min="6" max="9" width="28.42578125" customWidth="1"/>
+    <col min="6" max="9" width="28.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="95" t="s">
         <v>2</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30">
+    <row r="5" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="96" t="s">
         <v>7</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="30">
+    <row r="6" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="93" t="s">
         <v>12</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="30">
+    <row r="7" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="94" t="s">
         <v>17</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="60">
+    <row r="8" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="93" t="s">
         <v>22</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="45">
+    <row r="9" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="45">
+    <row r="10" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="7"/>
       <c r="B10" s="7" t="s">
         <v>32</v>
@@ -3124,7 +3124,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="45">
+    <row r="11" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="7"/>
       <c r="B11" s="7" t="s">
         <v>36</v>
@@ -3146,7 +3146,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="30">
+    <row r="12" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="7"/>
       <c r="B12" s="7" t="s">
         <v>42</v>
@@ -3168,7 +3168,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="75">
+    <row r="13" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="B13" s="7" t="s">
         <v>46</v>
@@ -3190,7 +3190,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="60">
+    <row r="14" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A14" s="7"/>
       <c r="B14" s="7" t="s">
         <v>50</v>
@@ -3210,7 +3210,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="93" t="s">
         <v>55</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="45">
+    <row r="16" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A16" s="94" t="s">
         <v>60</v>
       </c>
@@ -3250,7 +3250,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60">
+    <row r="17" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>65</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="2" t="s">
         <v>67</v>
@@ -3268,7 +3268,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="2" t="s">
         <v>69</v>
@@ -3277,7 +3277,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="2" t="s">
         <v>71</v>
@@ -3286,7 +3286,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="2" t="s">
         <v>73</v>
@@ -3295,7 +3295,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="2" t="s">
         <v>75</v>
@@ -3304,7 +3304,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="45">
+    <row r="24" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>77</v>
       </c>
@@ -3330,7 +3330,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>67</v>
       </c>
@@ -3342,7 +3342,7 @@
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
     </row>
-    <row r="26" spans="1:8" s="13" customFormat="1">
+    <row r="26" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>85</v>
       </c>
@@ -3358,7 +3358,7 @@
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
     </row>
-    <row r="27" spans="1:8" s="13" customFormat="1">
+    <row r="27" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
         <v>88</v>
@@ -3372,7 +3372,7 @@
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
     </row>
-    <row r="28" spans="1:8" s="13" customFormat="1">
+    <row r="28" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="11"/>
@@ -3384,7 +3384,7 @@
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>90</v>
       </c>
@@ -3398,7 +3398,7 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>85</v>
       </c>
@@ -3412,7 +3412,7 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
         <v>91</v>
@@ -3426,7 +3426,7 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="7"/>
@@ -3438,7 +3438,7 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>92</v>
       </c>
@@ -3450,7 +3450,7 @@
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" s="13" customFormat="1">
+    <row r="34" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>85</v>
       </c>
@@ -3466,7 +3466,7 @@
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="1:8" s="13" customFormat="1">
+    <row r="35" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="17"/>
       <c r="C35" s="2"/>
@@ -3478,7 +3478,7 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="1:8" s="13" customFormat="1">
+    <row r="36" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="17" t="s">
         <v>94</v>
@@ -3490,7 +3490,7 @@
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" s="13" customFormat="1">
+    <row r="37" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2" t="s">
         <v>95</v>
@@ -3504,7 +3504,7 @@
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="1:8" s="13" customFormat="1">
+    <row r="38" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -3516,7 +3516,7 @@
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="1:8" s="13" customFormat="1">
+    <row r="39" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2" t="s">
         <v>96</v>
@@ -3530,7 +3530,7 @@
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="1:8" s="13" customFormat="1">
+    <row r="40" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -3542,7 +3542,7 @@
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="1:8" s="13" customFormat="1">
+    <row r="41" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2" t="s">
         <v>97</v>
@@ -3556,7 +3556,7 @@
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="1:8" s="13" customFormat="1">
+    <row r="42" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -3568,7 +3568,7 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" s="13" customFormat="1">
+    <row r="43" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2" t="s">
         <v>98</v>
@@ -3582,7 +3582,7 @@
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="1:8" s="13" customFormat="1">
+    <row r="44" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -3594,7 +3594,7 @@
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="1:8" s="13" customFormat="1">
+    <row r="45" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="2" t="s">
         <v>99</v>
@@ -3608,7 +3608,7 @@
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="1:8" s="13" customFormat="1">
+    <row r="46" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -3620,7 +3620,7 @@
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="1:8" s="13" customFormat="1">
+    <row r="47" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="2" t="s">
         <v>100</v>
@@ -3634,7 +3634,7 @@
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="1:8" s="13" customFormat="1">
+    <row r="48" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -3646,7 +3646,7 @@
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="1:8" s="13" customFormat="1">
+    <row r="49" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2" t="s">
         <v>101</v>
@@ -3660,7 +3660,7 @@
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="1:8" s="13" customFormat="1">
+    <row r="50" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -3672,7 +3672,7 @@
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="1:8" s="13" customFormat="1">
+    <row r="51" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>102</v>
       </c>
@@ -3684,7 +3684,7 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
     </row>
-    <row r="52" spans="1:8" s="13" customFormat="1">
+    <row r="52" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>85</v>
       </c>
@@ -3698,7 +3698,7 @@
       <c r="G52" s="14"/>
       <c r="H52" s="14"/>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="1"/>
       <c r="B53" s="1" t="s">
         <v>103</v>
@@ -3712,7 +3712,7 @@
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -3724,7 +3724,7 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="1"/>
       <c r="B55" s="1" t="s">
         <v>105</v>
@@ -3736,7 +3736,7 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="1"/>
       <c r="B56" s="1" t="s">
         <v>106</v>
@@ -3750,7 +3750,7 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -3762,7 +3762,7 @@
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="1"/>
       <c r="B58" s="1" t="s">
         <v>107</v>
@@ -3776,7 +3776,7 @@
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -3788,7 +3788,7 @@
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -3800,7 +3800,7 @@
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>108</v>
       </c>
@@ -3814,7 +3814,7 @@
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>85</v>
       </c>
@@ -3828,7 +3828,7 @@
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -3840,7 +3840,7 @@
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -3852,7 +3852,7 @@
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2" t="s">
         <v>109</v>
@@ -3866,7 +3866,7 @@
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="2" t="s">
         <v>110</v>
@@ -3880,7 +3880,7 @@
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -3892,7 +3892,7 @@
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="2" t="s">
         <v>111</v>
@@ -3906,7 +3906,7 @@
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -3918,7 +3918,7 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="2" t="s">
         <v>112</v>
@@ -3932,7 +3932,7 @@
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -3944,7 +3944,7 @@
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -3956,7 +3956,7 @@
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2" t="s">
         <v>113</v>
@@ -3970,7 +3970,7 @@
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="2" t="s">
         <v>114</v>
@@ -3984,7 +3984,7 @@
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -3996,7 +3996,7 @@
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="2" t="s">
         <v>73</v>
@@ -4010,7 +4010,7 @@
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -4022,7 +4022,7 @@
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="1:8" ht="30">
+    <row r="78" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>115</v>
       </c>
@@ -4038,7 +4038,7 @@
       <c r="G78" s="1"/>
       <c r="H78" s="1"/>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
         <v>85</v>
       </c>
@@ -4052,7 +4052,7 @@
       <c r="G79" s="1"/>
       <c r="H79" s="1"/>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
         <v>85</v>
       </c>
@@ -4068,7 +4068,7 @@
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="7"/>
       <c r="B81" s="7"/>
       <c r="C81" s="1"/>
@@ -4080,7 +4080,7 @@
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="8" t="s">
         <v>60</v>
       </c>
@@ -4092,7 +4092,7 @@
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2" t="s">
         <v>118</v>
@@ -4106,7 +4106,7 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -4118,7 +4118,7 @@
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>85</v>
       </c>
@@ -4134,7 +4134,7 @@
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="1:8">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -4146,7 +4146,7 @@
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -4158,7 +4158,7 @@
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="2" t="s">
         <v>119</v>
@@ -4174,7 +4174,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>121</v>
       </c>
@@ -4188,7 +4188,7 @@
       <c r="G89" s="1"/>
       <c r="H89" s="1"/>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>85</v>
       </c>
@@ -4202,7 +4202,7 @@
       <c r="G90" s="1"/>
       <c r="H90" s="1"/>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -4214,7 +4214,7 @@
       <c r="G91" s="1"/>
       <c r="H91" s="1"/>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -4226,7 +4226,7 @@
       <c r="G92" s="1"/>
       <c r="H92" s="1"/>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -4238,7 +4238,7 @@
       <c r="G93" s="1"/>
       <c r="H93" s="1"/>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -4250,7 +4250,7 @@
       <c r="G94" s="1"/>
       <c r="H94" s="1"/>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" s="1"/>
       <c r="B95" s="1" t="s">
         <v>109</v>
@@ -4264,7 +4264,7 @@
       <c r="G95" s="1"/>
       <c r="H95" s="1"/>
     </row>
-    <row r="96" spans="1:8">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -4276,7 +4276,7 @@
       <c r="G96" s="1"/>
       <c r="H96" s="1"/>
     </row>
-    <row r="97" spans="1:8">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>122</v>
       </c>
@@ -4288,7 +4288,7 @@
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="1:8">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="2" t="s">
         <v>123</v>
@@ -4302,7 +4302,7 @@
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="1:8">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -4314,7 +4314,7 @@
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="1:8">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -4326,7 +4326,7 @@
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="1:8">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101" s="2"/>
       <c r="B101" s="2" t="s">
         <v>124</v>
@@ -4340,7 +4340,7 @@
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="1:8">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -4352,7 +4352,7 @@
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="1:8">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -4364,7 +4364,7 @@
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="1:8">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -4376,7 +4376,7 @@
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="1:8">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" s="2"/>
       <c r="B105" s="2" t="s">
         <v>125</v>
@@ -4390,7 +4390,7 @@
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="1:8">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -4402,7 +4402,7 @@
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="1:8">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -4414,7 +4414,7 @@
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="1:8">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>126</v>
       </c>
@@ -4426,7 +4426,7 @@
       <c r="G108" s="1"/>
       <c r="H108" s="1"/>
     </row>
-    <row r="109" spans="1:8">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>85</v>
       </c>
@@ -4442,7 +4442,7 @@
       <c r="G109" s="1"/>
       <c r="H109" s="1"/>
     </row>
-    <row r="110" spans="1:8">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -4454,7 +4454,7 @@
       <c r="G110" s="1"/>
       <c r="H110" s="1"/>
     </row>
-    <row r="111" spans="1:8">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A111" s="1"/>
       <c r="B111" s="1" t="s">
         <v>128</v>
@@ -4468,7 +4468,7 @@
       <c r="G111" s="1"/>
       <c r="H111" s="1"/>
     </row>
-    <row r="112" spans="1:8">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A112" s="1"/>
       <c r="B112" s="1" t="s">
         <v>129</v>
@@ -4482,7 +4482,7 @@
       <c r="G112" s="1"/>
       <c r="H112" s="1"/>
     </row>
-    <row r="114" spans="1:8" ht="30">
+    <row r="114" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A114" s="19" t="s">
         <v>130</v>
       </c>
@@ -4496,7 +4496,7 @@
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="1:8">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
         <v>131</v>
       </c>
@@ -4510,7 +4510,7 @@
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A116" s="3" t="s">
         <v>132</v>
       </c>
@@ -4524,7 +4524,7 @@
       <c r="G116" s="1"/>
       <c r="H116" s="1"/>
     </row>
-    <row r="117" spans="1:8">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>131</v>
       </c>
@@ -4538,7 +4538,7 @@
       <c r="G117" s="1"/>
       <c r="H117" s="1"/>
     </row>
-    <row r="118" spans="1:8">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
         <v>92</v>
       </c>
@@ -4552,7 +4552,7 @@
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="1:8">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -4564,7 +4564,7 @@
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="1:8">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
         <v>131</v>
       </c>
@@ -4580,7 +4580,7 @@
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="1:8">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -4592,7 +4592,7 @@
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="1:8">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A122" s="2"/>
       <c r="B122" s="2" t="s">
         <v>134</v>
@@ -4606,7 +4606,7 @@
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="1:8">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -4618,7 +4618,7 @@
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="1:8">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A124" s="2"/>
       <c r="B124" s="2" t="s">
         <v>135</v>
@@ -4632,7 +4632,7 @@
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="1:8">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -4644,7 +4644,7 @@
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="1:8">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A126" s="2"/>
       <c r="B126" s="2" t="s">
         <v>97</v>
@@ -4658,7 +4658,7 @@
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="1:8">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -4670,7 +4670,7 @@
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="1:8">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A128" s="2"/>
       <c r="B128" s="2" t="s">
         <v>93</v>
@@ -4684,7 +4684,7 @@
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="1:8">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -4696,7 +4696,7 @@
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="1:8">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -4708,7 +4708,7 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="1:8">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A131" s="2"/>
       <c r="B131" s="2" t="s">
         <v>136</v>
@@ -4722,7 +4722,7 @@
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="1:8">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -4734,7 +4734,7 @@
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="1:8">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A133" s="2"/>
       <c r="B133" s="2" t="s">
         <v>137</v>
@@ -4748,7 +4748,7 @@
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="1:8">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -4760,7 +4760,7 @@
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="1:8">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A135" s="2"/>
       <c r="B135" s="2" t="s">
         <v>138</v>
@@ -4774,7 +4774,7 @@
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="1:8">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -4786,7 +4786,7 @@
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="1:8">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A137" s="2"/>
       <c r="B137" s="2" t="s">
         <v>139</v>
@@ -4800,7 +4800,7 @@
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="1:8">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -4812,7 +4812,7 @@
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="1:8">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>90</v>
       </c>
@@ -4826,7 +4826,7 @@
       <c r="G139" s="1"/>
       <c r="H139" s="1"/>
     </row>
-    <row r="140" spans="1:8">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>131</v>
       </c>
@@ -4840,7 +4840,7 @@
       <c r="G140" s="1"/>
       <c r="H140" s="1"/>
     </row>
-    <row r="141" spans="1:8">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
         <v>140</v>
       </c>
@@ -4852,7 +4852,7 @@
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="1:8">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
         <v>131</v>
       </c>
@@ -4868,7 +4868,7 @@
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="1:8">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
@@ -4880,7 +4880,7 @@
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="1:8">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A144" s="2"/>
       <c r="B144" s="2" t="s">
         <v>142</v>
@@ -4894,7 +4894,7 @@
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="1:8">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -4906,7 +4906,7 @@
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="1:8">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A146" s="2"/>
       <c r="B146" s="2" t="s">
         <v>143</v>
@@ -4920,7 +4920,7 @@
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="1:8">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -4932,7 +4932,7 @@
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="1:8">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A148" s="2"/>
       <c r="B148" s="2" t="s">
         <v>144</v>
@@ -4946,7 +4946,7 @@
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="1:8">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -4958,7 +4958,7 @@
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="1:8">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A150" s="2"/>
       <c r="B150" s="2" t="s">
         <v>145</v>
@@ -4972,7 +4972,7 @@
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="1:8">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -4984,7 +4984,7 @@
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="1:8">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>146</v>
       </c>
@@ -4996,7 +4996,7 @@
       <c r="G152" s="1"/>
       <c r="H152" s="1"/>
     </row>
-    <row r="153" spans="1:8">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>131</v>
       </c>
@@ -5012,7 +5012,7 @@
       <c r="G153" s="1"/>
       <c r="H153" s="1"/>
     </row>
-    <row r="154" spans="1:8">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -5024,7 +5024,7 @@
       <c r="G154" s="1"/>
       <c r="H154" s="1"/>
     </row>
-    <row r="155" spans="1:8">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A155" s="1"/>
       <c r="B155" s="1" t="s">
         <v>147</v>
@@ -5038,7 +5038,7 @@
       <c r="G155" s="1"/>
       <c r="H155" s="1"/>
     </row>
-    <row r="156" spans="1:8">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -5050,7 +5050,7 @@
       <c r="G156" s="1"/>
       <c r="H156" s="1"/>
     </row>
-    <row r="157" spans="1:8">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A157" s="1"/>
       <c r="B157" s="1" t="s">
         <v>105</v>
@@ -5064,7 +5064,7 @@
       <c r="G157" s="1"/>
       <c r="H157" s="1"/>
     </row>
-    <row r="158" spans="1:8">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -5076,7 +5076,7 @@
       <c r="G158" s="1"/>
       <c r="H158" s="1"/>
     </row>
-    <row r="159" spans="1:8">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A159" s="1"/>
       <c r="B159" s="1" t="s">
         <v>106</v>
@@ -5090,7 +5090,7 @@
       <c r="G159" s="1"/>
       <c r="H159" s="1"/>
     </row>
-    <row r="160" spans="1:8">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -5102,7 +5102,7 @@
       <c r="G160" s="1"/>
       <c r="H160" s="1"/>
     </row>
-    <row r="161" spans="1:8">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A161" s="1"/>
       <c r="B161" s="1" t="s">
         <v>148</v>
@@ -5116,7 +5116,7 @@
       <c r="G161" s="1"/>
       <c r="H161" s="1"/>
     </row>
-    <row r="162" spans="1:8">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -5128,7 +5128,7 @@
       <c r="G162" s="1"/>
       <c r="H162" s="1"/>
     </row>
-    <row r="163" spans="1:8">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A163" s="1"/>
       <c r="B163" s="1" t="s">
         <v>149</v>
@@ -5142,7 +5142,7 @@
       <c r="G163" s="1"/>
       <c r="H163" s="1"/>
     </row>
-    <row r="164" spans="1:8">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -5154,7 +5154,7 @@
       <c r="G164" s="1"/>
       <c r="H164" s="1"/>
     </row>
-    <row r="165" spans="1:8">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A165" s="17" t="s">
         <v>126</v>
       </c>
@@ -5166,7 +5166,7 @@
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="1:8">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
         <v>131</v>
       </c>
@@ -5182,7 +5182,7 @@
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="1:8">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A167" s="17"/>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
@@ -5194,7 +5194,7 @@
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="1:8">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A168" s="2"/>
       <c r="B168" s="2" t="s">
         <v>151</v>
@@ -5208,7 +5208,7 @@
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="1:8">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
@@ -5220,7 +5220,7 @@
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="1:8">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A170" s="2"/>
       <c r="B170" s="2" t="s">
         <v>152</v>
@@ -5234,7 +5234,7 @@
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="1:8">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
@@ -5246,7 +5246,7 @@
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="1:8">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
         <v>153</v>
       </c>
@@ -5258,7 +5258,7 @@
       <c r="G172" s="1"/>
       <c r="H172" s="1"/>
     </row>
-    <row r="173" spans="1:8">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
         <v>131</v>
       </c>
@@ -5274,7 +5274,7 @@
       <c r="G173" s="1"/>
       <c r="H173" s="1"/>
     </row>
-    <row r="174" spans="1:8">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -5286,7 +5286,7 @@
       <c r="G174" s="1"/>
       <c r="H174" s="1"/>
     </row>
-    <row r="175" spans="1:8">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A175" s="1"/>
       <c r="B175" s="1" t="s">
         <v>155</v>
@@ -5300,7 +5300,7 @@
       <c r="G175" s="1"/>
       <c r="H175" s="1"/>
     </row>
-    <row r="176" spans="1:8">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
@@ -5312,7 +5312,7 @@
       <c r="G176" s="1"/>
       <c r="H176" s="1"/>
     </row>
-    <row r="177" spans="1:8">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A177" s="1"/>
       <c r="B177" s="1" t="s">
         <v>156</v>
@@ -5326,7 +5326,7 @@
       <c r="G177" s="1"/>
       <c r="H177" s="1"/>
     </row>
-    <row r="178" spans="1:8">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
@@ -5338,7 +5338,7 @@
       <c r="G178" s="1"/>
       <c r="H178" s="1"/>
     </row>
-    <row r="179" spans="1:8">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A179" s="1"/>
       <c r="B179" s="1" t="s">
         <v>157</v>
@@ -5352,7 +5352,7 @@
       <c r="G179" s="1"/>
       <c r="H179" s="1"/>
     </row>
-    <row r="180" spans="1:8">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
@@ -5364,7 +5364,7 @@
       <c r="G180" s="1"/>
       <c r="H180" s="1"/>
     </row>
-    <row r="181" spans="1:8">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A181" s="1"/>
       <c r="B181" s="1" t="s">
         <v>158</v>
@@ -5378,7 +5378,7 @@
       <c r="G181" s="1"/>
       <c r="H181" s="1"/>
     </row>
-    <row r="182" spans="1:8">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
@@ -5390,7 +5390,7 @@
       <c r="G182" s="1"/>
       <c r="H182" s="1"/>
     </row>
-    <row r="183" spans="1:8">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A183" s="1"/>
       <c r="B183" s="1" t="s">
         <v>159</v>
@@ -5404,7 +5404,7 @@
       <c r="G183" s="1"/>
       <c r="H183" s="1"/>
     </row>
-    <row r="184" spans="1:8">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
@@ -5416,7 +5416,7 @@
       <c r="G184" s="1"/>
       <c r="H184" s="1"/>
     </row>
-    <row r="185" spans="1:8">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
@@ -5428,7 +5428,7 @@
       <c r="G185" s="1"/>
       <c r="H185" s="1"/>
     </row>
-    <row r="186" spans="1:8">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
         <v>160</v>
       </c>
@@ -5444,7 +5444,7 @@
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="1:8">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
         <v>131</v>
       </c>
@@ -5458,7 +5458,7 @@
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="1:8">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A188" s="2"/>
       <c r="B188" s="2" t="s">
         <v>162</v>
@@ -5472,7 +5472,7 @@
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="1:8">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
@@ -5484,7 +5484,7 @@
       <c r="G189" s="2"/>
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="1:8">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A190" s="2"/>
       <c r="B190" s="2" t="s">
         <v>163</v>
@@ -5498,7 +5498,7 @@
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="1:8">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
@@ -5510,7 +5510,7 @@
       <c r="G191" s="2"/>
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="1:8">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A192" s="2"/>
       <c r="B192" s="2" t="s">
         <v>121</v>
@@ -5524,7 +5524,7 @@
       <c r="G192" s="2"/>
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="1:8">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="2"/>
@@ -5536,7 +5536,7 @@
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="1:8">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
         <v>164</v>
       </c>
@@ -5552,7 +5552,7 @@
       <c r="G194" s="1"/>
       <c r="H194" s="1"/>
     </row>
-    <row r="195" spans="1:8">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
@@ -5564,7 +5564,7 @@
       <c r="G195" s="1"/>
       <c r="H195" s="1"/>
     </row>
-    <row r="196" spans="1:8">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A196" s="1"/>
       <c r="B196" s="1" t="s">
         <v>165</v>
@@ -5578,7 +5578,7 @@
       <c r="G196" s="1"/>
       <c r="H196" s="1"/>
     </row>
-    <row r="197" spans="1:8">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
@@ -5590,7 +5590,7 @@
       <c r="G197" s="1"/>
       <c r="H197" s="1"/>
     </row>
-    <row r="198" spans="1:8">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A198" s="1"/>
       <c r="B198" s="1" t="s">
         <v>155</v>
@@ -5604,7 +5604,7 @@
       <c r="G198" s="1"/>
       <c r="H198" s="1"/>
     </row>
-    <row r="199" spans="1:8">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
@@ -5616,7 +5616,7 @@
       <c r="G199" s="1"/>
       <c r="H199" s="1"/>
     </row>
-    <row r="200" spans="1:8">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A200" s="1"/>
       <c r="B200" s="1" t="s">
         <v>153</v>
@@ -5630,7 +5630,7 @@
       <c r="G200" s="1"/>
       <c r="H200" s="1"/>
     </row>
-    <row r="201" spans="1:8">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
@@ -5642,7 +5642,7 @@
       <c r="G201" s="1"/>
       <c r="H201" s="1"/>
     </row>
-    <row r="202" spans="1:8">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A202" s="1"/>
       <c r="B202" s="1" t="s">
         <v>166</v>
@@ -5656,7 +5656,7 @@
       <c r="G202" s="1"/>
       <c r="H202" s="1"/>
     </row>
-    <row r="203" spans="1:8">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
@@ -5668,7 +5668,7 @@
       <c r="G203" s="1"/>
       <c r="H203" s="1"/>
     </row>
-    <row r="204" spans="1:8">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A204" s="1"/>
       <c r="B204" s="1" t="s">
         <v>167</v>
@@ -5682,7 +5682,7 @@
       <c r="G204" s="1"/>
       <c r="H204" s="1"/>
     </row>
-    <row r="205" spans="1:8">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
@@ -5694,7 +5694,7 @@
       <c r="G205" s="1"/>
       <c r="H205" s="1"/>
     </row>
-    <row r="206" spans="1:8">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A206" s="1"/>
       <c r="B206" s="1" t="s">
         <v>168</v>
@@ -5708,7 +5708,7 @@
       <c r="G206" s="1"/>
       <c r="H206" s="1"/>
     </row>
-    <row r="207" spans="1:8">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
@@ -5720,7 +5720,7 @@
       <c r="G207" s="1"/>
       <c r="H207" s="1"/>
     </row>
-    <row r="208" spans="1:8">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A208" s="1"/>
       <c r="B208" s="1" t="s">
         <v>169</v>
@@ -5734,7 +5734,7 @@
       <c r="G208" s="1"/>
       <c r="H208" s="1"/>
     </row>
-    <row r="209" spans="1:8">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
@@ -5746,7 +5746,7 @@
       <c r="G209" s="1"/>
       <c r="H209" s="1"/>
     </row>
-    <row r="210" spans="1:8">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A210" s="1"/>
       <c r="B210" s="1" t="s">
         <v>170</v>
@@ -5760,7 +5760,7 @@
       <c r="G210" s="1"/>
       <c r="H210" s="1"/>
     </row>
-    <row r="211" spans="1:8">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
@@ -5772,7 +5772,7 @@
       <c r="G211" s="1"/>
       <c r="H211" s="1"/>
     </row>
-    <row r="212" spans="1:8">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A212" s="2" t="s">
         <v>171</v>
       </c>
@@ -5788,7 +5788,7 @@
       <c r="G212" s="2"/>
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="1:8">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
       <c r="C213" s="2"/>
@@ -5800,7 +5800,7 @@
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="1:8">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A214" s="2" t="s">
         <v>131</v>
       </c>
@@ -5816,7 +5816,7 @@
       <c r="G214" s="2"/>
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="1:8">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A215" s="2"/>
       <c r="B215" s="2"/>
       <c r="C215" s="2"/>
@@ -5828,7 +5828,7 @@
       <c r="G215" s="2"/>
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="1:8">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A216" s="2" t="s">
         <v>164</v>
       </c>
@@ -5844,7 +5844,7 @@
       <c r="G216" s="2"/>
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="1:8">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A217" s="2"/>
       <c r="B217" s="2"/>
       <c r="C217" s="2"/>
@@ -5856,7 +5856,7 @@
       <c r="G217" s="2"/>
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="1:8">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A218" s="2"/>
       <c r="B218" s="2"/>
       <c r="C218" s="2"/>
@@ -5868,7 +5868,7 @@
       <c r="G218" s="2"/>
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="1:8">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A219" s="2"/>
       <c r="B219" s="2" t="s">
         <v>171</v>
@@ -5882,7 +5882,7 @@
       <c r="G219" s="2"/>
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="1:8">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A220" s="2"/>
       <c r="B220" s="2"/>
       <c r="C220" s="2"/>
@@ -5894,7 +5894,7 @@
       <c r="G220" s="2"/>
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="1:8">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A221" s="2"/>
       <c r="B221" s="2"/>
       <c r="C221" s="2"/>
@@ -5906,7 +5906,7 @@
       <c r="G221" s="2"/>
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="1:8">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A222" s="1" t="s">
         <v>175</v>
       </c>
@@ -5920,7 +5920,7 @@
       <c r="G222" s="1"/>
       <c r="H222" s="1"/>
     </row>
-    <row r="223" spans="1:8">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="s">
         <v>131</v>
       </c>
@@ -5934,7 +5934,7 @@
       <c r="G223" s="1"/>
       <c r="H223" s="1"/>
     </row>
-    <row r="224" spans="1:8">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A224" s="1"/>
       <c r="B224" s="1" t="s">
         <v>176</v>
@@ -5948,7 +5948,7 @@
       <c r="G224" s="1"/>
       <c r="H224" s="1"/>
     </row>
-    <row r="225" spans="1:8">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A225" s="1"/>
       <c r="B225" s="1"/>
       <c r="C225" s="1"/>
@@ -5960,7 +5960,7 @@
       <c r="G225" s="1"/>
       <c r="H225" s="1"/>
     </row>
-    <row r="226" spans="1:8">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A226" s="2" t="s">
         <v>177</v>
       </c>
@@ -5976,7 +5976,7 @@
       <c r="G226" s="2"/>
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="1:8">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A227" s="2"/>
       <c r="B227" s="2"/>
       <c r="C227" s="2"/>
@@ -5988,7 +5988,7 @@
       <c r="G227" s="2"/>
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="1:8">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A228" s="2" t="s">
         <v>131</v>
       </c>
@@ -6004,7 +6004,7 @@
       <c r="G228" s="2"/>
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="1:8">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A229" s="2"/>
       <c r="B229" s="2"/>
       <c r="C229" s="2"/>
@@ -6016,7 +6016,7 @@
       <c r="G229" s="2"/>
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="1:8">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A230" s="2"/>
       <c r="B230" s="2"/>
       <c r="C230" s="2"/>
@@ -6028,7 +6028,7 @@
       <c r="G230" s="2"/>
       <c r="H230" s="2"/>
     </row>
-    <row r="231" spans="1:8">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A231" s="2"/>
       <c r="B231" s="2"/>
       <c r="C231" s="2"/>
@@ -6040,7 +6040,7 @@
       <c r="G231" s="2"/>
       <c r="H231" s="2"/>
     </row>
-    <row r="232" spans="1:8">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
         <v>180</v>
       </c>
@@ -6052,7 +6052,7 @@
       <c r="G232" s="1"/>
       <c r="H232" s="1"/>
     </row>
-    <row r="233" spans="1:8">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A233" s="1"/>
       <c r="B233" s="1" t="s">
         <v>181</v>
@@ -6066,7 +6066,7 @@
       <c r="G233" s="1"/>
       <c r="H233" s="1"/>
     </row>
-    <row r="234" spans="1:8">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A234" s="1"/>
       <c r="B234" s="1"/>
       <c r="C234" s="1"/>
@@ -6078,7 +6078,7 @@
       <c r="G234" s="1"/>
       <c r="H234" s="1"/>
     </row>
-    <row r="235" spans="1:8">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
         <v>131</v>
       </c>
@@ -6094,7 +6094,7 @@
       <c r="G235" s="1"/>
       <c r="H235" s="1"/>
     </row>
-    <row r="236" spans="1:8">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A236" s="1"/>
       <c r="B236" s="1"/>
       <c r="C236" s="1"/>
@@ -6106,7 +6106,7 @@
       <c r="G236" s="1"/>
       <c r="H236" s="1"/>
     </row>
-    <row r="237" spans="1:8">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A237" s="1"/>
       <c r="B237" s="1"/>
       <c r="C237" s="1"/>
@@ -6118,7 +6118,7 @@
       <c r="G237" s="1"/>
       <c r="H237" s="1"/>
     </row>
-    <row r="238" spans="1:8">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A238" s="1"/>
       <c r="B238" s="1" t="s">
         <v>183</v>
@@ -6132,7 +6132,7 @@
       <c r="G238" s="1"/>
       <c r="H238" s="1"/>
     </row>
-    <row r="239" spans="1:8">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A239" s="1"/>
       <c r="B239" s="1"/>
       <c r="C239" s="1"/>
@@ -6144,7 +6144,7 @@
       <c r="G239" s="1"/>
       <c r="H239" s="1"/>
     </row>
-    <row r="240" spans="1:8">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A240" s="1"/>
       <c r="B240" s="1"/>
       <c r="C240" s="1"/>
@@ -6156,7 +6156,7 @@
       <c r="G240" s="1"/>
       <c r="H240" s="1"/>
     </row>
-    <row r="241" spans="1:8">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A241" s="2" t="s">
         <v>36</v>
       </c>
@@ -6170,7 +6170,7 @@
       <c r="G241" s="2"/>
       <c r="H241" s="2"/>
     </row>
-    <row r="242" spans="1:8">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A242" s="2" t="s">
         <v>131</v>
       </c>
@@ -6184,7 +6184,7 @@
       <c r="G242" s="2"/>
       <c r="H242" s="2"/>
     </row>
-    <row r="243" spans="1:8">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
         <v>184</v>
       </c>
@@ -6198,7 +6198,7 @@
       <c r="G243" s="1"/>
       <c r="H243" s="1"/>
     </row>
-    <row r="244" spans="1:8">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="s">
         <v>131</v>
       </c>
@@ -6214,7 +6214,7 @@
       <c r="G244" s="1"/>
       <c r="H244" s="1"/>
     </row>
-    <row r="245" spans="1:8">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A245" s="1"/>
       <c r="B245" s="1"/>
       <c r="C245" s="1"/>
@@ -6436,28 +6436,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AMJ186"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="2" max="2" width="12.5" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" style="22" customWidth="1"/>
-    <col min="6" max="6" width="43.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" customWidth="1"/>
-    <col min="9" max="9" width="6.85546875" customWidth="1"/>
-    <col min="10" max="10" width="36.140625" customWidth="1"/>
-    <col min="11" max="11" width="37.7109375" customWidth="1"/>
-    <col min="12" max="12" width="45.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="5" max="5" width="18.5" style="22" customWidth="1"/>
+    <col min="6" max="6" width="43.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.5" customWidth="1"/>
+    <col min="9" max="9" width="6.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.1640625" customWidth="1"/>
+    <col min="11" max="11" width="37.6640625" customWidth="1"/>
+    <col min="12" max="12" width="45.1640625" customWidth="1"/>
     <col min="13" max="13" width="41" customWidth="1"/>
-    <col min="14" max="14" width="32.7109375" customWidth="1"/>
+    <col min="14" max="14" width="32.6640625" customWidth="1"/>
     <col min="15" max="15" width="32" customWidth="1"/>
-    <col min="16" max="16" width="63.7109375" customWidth="1"/>
-    <col min="1024" max="1024" width="11.42578125" customWidth="1"/>
+    <col min="16" max="16" width="63.6640625" customWidth="1"/>
+    <col min="1024" max="1024" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="30">
+    <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>186</v>
       </c>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="Q1" s="24"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="25">
         <v>2</v>
       </c>
@@ -6536,7 +6536,7 @@
       <c r="O2" s="5"/>
       <c r="R2" s="13"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="28">
         <v>4</v>
       </c>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="Q3" s="35"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="28">
         <v>5</v>
       </c>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="Q4" s="35"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="36">
         <v>6</v>
       </c>
@@ -6661,7 +6661,7 @@
       </c>
       <c r="Q5" s="35"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="36">
         <v>7</v>
       </c>
@@ -6704,7 +6704,7 @@
       </c>
       <c r="Q6" s="42"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="28">
         <v>210</v>
       </c>
@@ -6737,7 +6737,7 @@
       </c>
       <c r="Q7" s="35"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="28">
         <v>8</v>
       </c>
@@ -6774,7 +6774,7 @@
       </c>
       <c r="Q8" s="35"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="28">
         <v>9</v>
       </c>
@@ -6817,7 +6817,7 @@
       </c>
       <c r="Q9" s="42"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="28"/>
       <c r="B10" s="21"/>
       <c r="C10" s="28">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="Q10" s="42"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="28"/>
       <c r="B11" s="21"/>
       <c r="C11" s="28">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="Q11" s="42"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="28">
         <v>10</v>
       </c>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="Q12" s="35"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="28">
         <v>11</v>
       </c>
@@ -6955,7 +6955,7 @@
       </c>
       <c r="Q13" s="35"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="28">
         <v>12</v>
       </c>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="Q14" s="35"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="28"/>
       <c r="B15" s="21"/>
       <c r="C15" s="28">
@@ -7029,7 +7029,7 @@
       </c>
       <c r="Q15" s="35"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="28">
         <v>13</v>
       </c>
@@ -7070,7 +7070,7 @@
       </c>
       <c r="Q16" s="35"/>
     </row>
-    <row r="17" spans="1:1024">
+    <row r="17" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="28">
         <v>14</v>
       </c>
@@ -7113,7 +7113,7 @@
       </c>
       <c r="Q17" s="35"/>
     </row>
-    <row r="18" spans="1:1024">
+    <row r="18" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="28">
         <v>16</v>
       </c>
@@ -7156,7 +7156,7 @@
       </c>
       <c r="Q18" s="35"/>
     </row>
-    <row r="19" spans="1:1024">
+    <row r="19" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="28">
         <v>17</v>
       </c>
@@ -7199,7 +7199,7 @@
       </c>
       <c r="Q19" s="35"/>
     </row>
-    <row r="20" spans="1:1024">
+    <row r="20" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="28">
         <v>15</v>
       </c>
@@ -7242,7 +7242,7 @@
       </c>
       <c r="Q20" s="35"/>
     </row>
-    <row r="21" spans="1:1024" s="72" customFormat="1">
+    <row r="21" spans="1:1024" s="72" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="66">
         <v>201</v>
       </c>
@@ -7273,7 +7273,7 @@
       </c>
       <c r="Q21" s="71"/>
     </row>
-    <row r="22" spans="1:1024">
+    <row r="22" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="36">
         <v>18</v>
       </c>
@@ -7312,7 +7312,7 @@
       </c>
       <c r="Q22" s="35"/>
     </row>
-    <row r="23" spans="1:1024">
+    <row r="23" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A23" s="36">
         <v>19</v>
       </c>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="Q23" s="42"/>
     </row>
-    <row r="24" spans="1:1024">
+    <row r="24" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A24" s="36"/>
       <c r="B24" s="3"/>
       <c r="C24" s="36">
@@ -7386,7 +7386,7 @@
       </c>
       <c r="Q24" s="42"/>
     </row>
-    <row r="25" spans="1:1024">
+    <row r="25" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A25" s="36"/>
       <c r="B25" s="3"/>
       <c r="C25" s="36">
@@ -7417,7 +7417,7 @@
       </c>
       <c r="Q25" s="42"/>
     </row>
-    <row r="26" spans="1:1024">
+    <row r="26" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="36">
         <v>20</v>
       </c>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="Q26" s="35"/>
     </row>
-    <row r="27" spans="1:1024">
+    <row r="27" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="36">
         <v>21</v>
       </c>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="Q27" s="35"/>
     </row>
-    <row r="28" spans="1:1024">
+    <row r="28" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="36"/>
       <c r="B28" s="3"/>
       <c r="C28" s="36">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="Q28" s="35"/>
     </row>
-    <row r="29" spans="1:1024">
+    <row r="29" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A29" s="36">
         <v>22</v>
       </c>
@@ -7567,7 +7567,7 @@
       </c>
       <c r="Q29" s="42"/>
     </row>
-    <row r="30" spans="1:1024">
+    <row r="30" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A30" s="36"/>
       <c r="B30" s="3"/>
       <c r="C30" s="36">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="Q30" s="42"/>
     </row>
-    <row r="31" spans="1:1024">
+    <row r="31" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A31" s="36"/>
       <c r="B31" s="3"/>
       <c r="C31" s="36">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="Q31" s="42"/>
     </row>
-    <row r="32" spans="1:1024" s="85" customFormat="1">
+    <row r="32" spans="1:1024" s="85" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="50">
         <v>211</v>
       </c>
@@ -7663,7 +7663,7 @@
       <c r="Q32" s="84"/>
       <c r="AMJ32" s="86"/>
     </row>
-    <row r="33" spans="1:1024" s="85" customFormat="1">
+    <row r="33" spans="1:1024" s="85" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="50">
         <v>39</v>
       </c>
@@ -7699,7 +7699,7 @@
       <c r="Q33" s="84"/>
       <c r="AMJ33" s="86"/>
     </row>
-    <row r="34" spans="1:1024" s="55" customFormat="1">
+    <row r="34" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="50">
         <v>40</v>
       </c>
@@ -7743,7 +7743,7 @@
       <c r="Q34" s="57"/>
       <c r="AMJ34"/>
     </row>
-    <row r="35" spans="1:1024" s="55" customFormat="1">
+    <row r="35" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="50"/>
       <c r="B35" s="51"/>
       <c r="C35" s="50">
@@ -7775,7 +7775,7 @@
       <c r="Q35" s="57"/>
       <c r="AMJ35"/>
     </row>
-    <row r="36" spans="1:1024" s="55" customFormat="1">
+    <row r="36" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="50"/>
       <c r="B36" s="51"/>
       <c r="C36" s="50">
@@ -7807,7 +7807,7 @@
       <c r="Q36" s="57"/>
       <c r="AMJ36"/>
     </row>
-    <row r="37" spans="1:1024" s="55" customFormat="1">
+    <row r="37" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="50">
         <v>41</v>
       </c>
@@ -7849,7 +7849,7 @@
       <c r="Q37" s="57"/>
       <c r="AMJ37"/>
     </row>
-    <row r="38" spans="1:1024" s="55" customFormat="1">
+    <row r="38" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="50"/>
       <c r="B38" s="51"/>
       <c r="C38" s="50">
@@ -7881,7 +7881,7 @@
       <c r="Q38" s="57"/>
       <c r="AMJ38"/>
     </row>
-    <row r="39" spans="1:1024" s="55" customFormat="1">
+    <row r="39" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="50">
         <v>42</v>
       </c>
@@ -7923,7 +7923,7 @@
       <c r="Q39" s="57"/>
       <c r="AMJ39"/>
     </row>
-    <row r="40" spans="1:1024" s="80" customFormat="1">
+    <row r="40" spans="1:1024" s="80" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="73">
         <v>202</v>
       </c>
@@ -7953,7 +7953,7 @@
       <c r="Q40" s="79"/>
       <c r="AMJ40" s="81"/>
     </row>
-    <row r="41" spans="1:1024" s="55" customFormat="1">
+    <row r="41" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="28">
         <v>23</v>
       </c>
@@ -7993,7 +7993,7 @@
       <c r="Q41" s="54"/>
       <c r="AMJ41"/>
     </row>
-    <row r="42" spans="1:1024" s="55" customFormat="1">
+    <row r="42" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="28"/>
       <c r="B42" s="21"/>
       <c r="C42" s="28">
@@ -8025,7 +8025,7 @@
       <c r="Q42" s="54"/>
       <c r="AMJ42"/>
     </row>
-    <row r="43" spans="1:1024" s="55" customFormat="1">
+    <row r="43" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="28"/>
       <c r="B43" s="21"/>
       <c r="C43" s="28">
@@ -8061,7 +8061,7 @@
       <c r="Q43" s="54"/>
       <c r="AMJ43"/>
     </row>
-    <row r="44" spans="1:1024" s="55" customFormat="1">
+    <row r="44" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="28"/>
       <c r="B44" s="21"/>
       <c r="C44" s="28">
@@ -8099,7 +8099,7 @@
       <c r="Q44" s="54"/>
       <c r="AMJ44"/>
     </row>
-    <row r="45" spans="1:1024" s="55" customFormat="1">
+    <row r="45" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="28">
         <v>24</v>
       </c>
@@ -8143,7 +8143,7 @@
       <c r="Q45" s="54"/>
       <c r="AMJ45"/>
     </row>
-    <row r="46" spans="1:1024" s="55" customFormat="1">
+    <row r="46" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="28">
         <v>25</v>
       </c>
@@ -8187,7 +8187,7 @@
       <c r="Q46" s="54"/>
       <c r="AMJ46"/>
     </row>
-    <row r="47" spans="1:1024" s="55" customFormat="1">
+    <row r="47" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="28"/>
       <c r="B47" s="21"/>
       <c r="C47" s="28">
@@ -8219,7 +8219,7 @@
       <c r="Q47" s="54"/>
       <c r="AMJ47"/>
     </row>
-    <row r="48" spans="1:1024" s="55" customFormat="1">
+    <row r="48" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="28"/>
       <c r="B48" s="21"/>
       <c r="C48" s="28">
@@ -8251,7 +8251,7 @@
       <c r="Q48" s="54"/>
       <c r="AMJ48"/>
     </row>
-    <row r="49" spans="1:1024" s="55" customFormat="1">
+    <row r="49" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="28">
         <v>26</v>
       </c>
@@ -8296,7 +8296,7 @@
       </c>
       <c r="AMJ49"/>
     </row>
-    <row r="50" spans="1:1024" s="55" customFormat="1">
+    <row r="50" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="28"/>
       <c r="B50" s="21"/>
       <c r="C50" s="28">
@@ -8327,7 +8327,7 @@
       </c>
       <c r="AMJ50"/>
     </row>
-    <row r="51" spans="1:1024" s="55" customFormat="1">
+    <row r="51" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="28"/>
       <c r="B51" s="21"/>
       <c r="C51" s="28">
@@ -8361,7 +8361,7 @@
       <c r="Q51" s="54"/>
       <c r="AMJ51"/>
     </row>
-    <row r="52" spans="1:1024" s="55" customFormat="1">
+    <row r="52" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="28">
         <v>27</v>
       </c>
@@ -8405,7 +8405,7 @@
       <c r="Q52" s="54"/>
       <c r="AMJ52"/>
     </row>
-    <row r="53" spans="1:1024" s="55" customFormat="1">
+    <row r="53" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="28">
         <v>28</v>
       </c>
@@ -8449,7 +8449,7 @@
       <c r="Q53" s="54"/>
       <c r="AMJ53"/>
     </row>
-    <row r="54" spans="1:1024" s="55" customFormat="1">
+    <row r="54" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="28"/>
       <c r="B54" s="21"/>
       <c r="C54" s="28">
@@ -8481,7 +8481,7 @@
       <c r="Q54" s="54"/>
       <c r="AMJ54"/>
     </row>
-    <row r="55" spans="1:1024" s="55" customFormat="1">
+    <row r="55" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="28"/>
       <c r="B55" s="21"/>
       <c r="C55" s="28">
@@ -8513,7 +8513,7 @@
       <c r="Q55" s="54"/>
       <c r="AMJ55"/>
     </row>
-    <row r="56" spans="1:1024" s="55" customFormat="1" ht="30">
+    <row r="56" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="36">
         <v>212</v>
       </c>
@@ -8547,7 +8547,7 @@
       <c r="Q56" s="54"/>
       <c r="AMJ56"/>
     </row>
-    <row r="57" spans="1:1024" s="55" customFormat="1" ht="30">
+    <row r="57" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="36">
         <v>29</v>
       </c>
@@ -8589,7 +8589,7 @@
       <c r="Q57" s="54"/>
       <c r="AMJ57"/>
     </row>
-    <row r="58" spans="1:1024" s="55" customFormat="1">
+    <row r="58" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="36">
         <v>30</v>
       </c>
@@ -8631,7 +8631,7 @@
       <c r="Q58" s="57"/>
       <c r="AMJ58"/>
     </row>
-    <row r="59" spans="1:1024" s="55" customFormat="1">
+    <row r="59" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="36"/>
       <c r="B59" s="3"/>
       <c r="C59" s="36">
@@ -8663,7 +8663,7 @@
       <c r="Q59" s="57"/>
       <c r="AMJ59"/>
     </row>
-    <row r="60" spans="1:1024" s="55" customFormat="1">
+    <row r="60" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="50">
         <v>34</v>
       </c>
@@ -8711,7 +8711,7 @@
       <c r="Q60" s="54"/>
       <c r="AMJ60"/>
     </row>
-    <row r="61" spans="1:1024" s="55" customFormat="1">
+    <row r="61" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="50"/>
       <c r="B61" s="51"/>
       <c r="C61" s="50">
@@ -8743,7 +8743,7 @@
       <c r="Q61" s="54"/>
       <c r="AMJ61"/>
     </row>
-    <row r="62" spans="1:1024" s="55" customFormat="1">
+    <row r="62" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="50"/>
       <c r="B62" s="51"/>
       <c r="C62" s="50">
@@ -8775,7 +8775,7 @@
       <c r="Q62" s="54"/>
       <c r="AMJ62"/>
     </row>
-    <row r="63" spans="1:1024" s="55" customFormat="1">
+    <row r="63" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="50"/>
       <c r="B63" s="51"/>
       <c r="C63" s="50">
@@ -8809,7 +8809,7 @@
       <c r="Q63" s="54"/>
       <c r="AMJ63"/>
     </row>
-    <row r="64" spans="1:1024" s="55" customFormat="1">
+    <row r="64" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="50"/>
       <c r="B64" s="51"/>
       <c r="C64" s="50">
@@ -8847,7 +8847,7 @@
       <c r="Q64" s="57"/>
       <c r="AMJ64"/>
     </row>
-    <row r="65" spans="1:1024" s="55" customFormat="1">
+    <row r="65" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="28">
         <v>31</v>
       </c>
@@ -8879,7 +8879,7 @@
       <c r="Q65" s="54"/>
       <c r="AMJ65"/>
     </row>
-    <row r="66" spans="1:1024" s="55" customFormat="1">
+    <row r="66" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="28">
         <v>32</v>
       </c>
@@ -8921,7 +8921,7 @@
       <c r="Q66" s="54"/>
       <c r="AMJ66"/>
     </row>
-    <row r="67" spans="1:1024" s="55" customFormat="1">
+    <row r="67" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="28"/>
       <c r="B67" s="21"/>
       <c r="C67" s="28">
@@ -8953,7 +8953,7 @@
       <c r="Q67" s="54"/>
       <c r="AMJ67"/>
     </row>
-    <row r="68" spans="1:1024" s="55" customFormat="1">
+    <row r="68" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A68" s="28"/>
       <c r="B68" s="21"/>
       <c r="C68" s="28">
@@ -8991,7 +8991,7 @@
       <c r="Q68" s="57"/>
       <c r="AMJ68"/>
     </row>
-    <row r="69" spans="1:1024" s="55" customFormat="1">
+    <row r="69" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="28">
         <v>33</v>
       </c>
@@ -9033,7 +9033,7 @@
       <c r="Q69" s="54"/>
       <c r="AMJ69"/>
     </row>
-    <row r="70" spans="1:1024" s="55" customFormat="1">
+    <row r="70" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="36">
         <v>35</v>
       </c>
@@ -9067,7 +9067,7 @@
       <c r="Q70" s="54"/>
       <c r="AMJ70"/>
     </row>
-    <row r="71" spans="1:1024" s="55" customFormat="1">
+    <row r="71" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="36">
         <v>36</v>
       </c>
@@ -9111,7 +9111,7 @@
       <c r="Q71" s="57"/>
       <c r="AMJ71"/>
     </row>
-    <row r="72" spans="1:1024" s="55" customFormat="1">
+    <row r="72" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="36"/>
       <c r="B72" s="3"/>
       <c r="C72" s="36">
@@ -9143,7 +9143,7 @@
       <c r="Q72" s="57"/>
       <c r="AMJ72"/>
     </row>
-    <row r="73" spans="1:1024" s="55" customFormat="1">
+    <row r="73" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="36"/>
       <c r="B73" s="3"/>
       <c r="C73" s="36">
@@ -9175,7 +9175,7 @@
       <c r="Q73" s="57"/>
       <c r="AMJ73"/>
     </row>
-    <row r="74" spans="1:1024" s="55" customFormat="1">
+    <row r="74" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="36">
         <v>37</v>
       </c>
@@ -9215,7 +9215,7 @@
       <c r="Q74" s="57"/>
       <c r="AMJ74"/>
     </row>
-    <row r="75" spans="1:1024" s="55" customFormat="1">
+    <row r="75" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="36"/>
       <c r="B75" s="3"/>
       <c r="C75" s="36">
@@ -9247,7 +9247,7 @@
       <c r="Q75" s="57"/>
       <c r="AMJ75"/>
     </row>
-    <row r="76" spans="1:1024" s="55" customFormat="1">
+    <row r="76" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="36"/>
       <c r="B76" s="3"/>
       <c r="C76" s="36">
@@ -9279,7 +9279,7 @@
       <c r="Q76" s="57"/>
       <c r="AMJ76"/>
     </row>
-    <row r="77" spans="1:1024" s="55" customFormat="1">
+    <row r="77" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A77" s="36"/>
       <c r="B77" s="3"/>
       <c r="C77" s="36">
@@ -9311,7 +9311,7 @@
       <c r="Q77" s="54"/>
       <c r="AMJ77"/>
     </row>
-    <row r="78" spans="1:1024" s="55" customFormat="1">
+    <row r="78" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="36">
         <v>38</v>
       </c>
@@ -9355,7 +9355,7 @@
       <c r="Q78" s="57"/>
       <c r="AMJ78"/>
     </row>
-    <row r="79" spans="1:1024" s="55" customFormat="1">
+    <row r="79" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="36"/>
       <c r="B79" s="3"/>
       <c r="C79" s="36">
@@ -9387,7 +9387,7 @@
       <c r="Q79" s="57"/>
       <c r="AMJ79"/>
     </row>
-    <row r="80" spans="1:1024">
+    <row r="80" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A80" s="61">
         <v>43</v>
       </c>
@@ -9414,7 +9414,7 @@
       <c r="N80" s="63"/>
       <c r="Q80" s="42"/>
     </row>
-    <row r="81" spans="1:17">
+    <row r="81" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" s="28">
         <v>44</v>
       </c>
@@ -9453,7 +9453,7 @@
       </c>
       <c r="Q81" s="42"/>
     </row>
-    <row r="82" spans="1:17">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A82" s="36">
         <v>45</v>
       </c>
@@ -9490,7 +9490,7 @@
       </c>
       <c r="Q82" s="42"/>
     </row>
-    <row r="83" spans="1:17">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A83" s="28">
         <v>204</v>
       </c>
@@ -9521,7 +9521,7 @@
       </c>
       <c r="Q83" s="42"/>
     </row>
-    <row r="84" spans="1:17">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A84" s="28">
         <v>46</v>
       </c>
@@ -9558,7 +9558,7 @@
       </c>
       <c r="Q84" s="42"/>
     </row>
-    <row r="85" spans="1:17">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A85" s="28">
         <v>47</v>
       </c>
@@ -9597,7 +9597,7 @@
       </c>
       <c r="Q85" s="42"/>
     </row>
-    <row r="86" spans="1:17">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A86" s="28">
         <v>48</v>
       </c>
@@ -9636,7 +9636,7 @@
       </c>
       <c r="Q86" s="42"/>
     </row>
-    <row r="87" spans="1:17">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A87" s="28">
         <v>49</v>
       </c>
@@ -9675,7 +9675,7 @@
       </c>
       <c r="Q87" s="42"/>
     </row>
-    <row r="88" spans="1:17">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A88" s="28">
         <v>50</v>
       </c>
@@ -9714,7 +9714,7 @@
       </c>
       <c r="Q88" s="42"/>
     </row>
-    <row r="89" spans="1:17">
+    <row r="89" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A89" s="28">
         <v>54</v>
       </c>
@@ -9755,7 +9755,7 @@
       </c>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" spans="1:17">
+    <row r="90" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A90" s="28">
         <v>55</v>
       </c>
@@ -9796,7 +9796,7 @@
       </c>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" spans="1:17">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A91" s="36">
         <v>56</v>
       </c>
@@ -9837,7 +9837,7 @@
       </c>
       <c r="Q91" s="42"/>
     </row>
-    <row r="92" spans="1:17">
+    <row r="92" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A92" s="28">
         <v>57</v>
       </c>
@@ -9868,7 +9868,7 @@
       </c>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" spans="1:17">
+    <row r="93" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A93" s="28">
         <v>58</v>
       </c>
@@ -9907,7 +9907,7 @@
       </c>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" spans="1:17">
+    <row r="94" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A94" s="28">
         <v>59</v>
       </c>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" spans="1:17">
+    <row r="95" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A95" s="28">
         <v>60</v>
       </c>
@@ -9989,7 +9989,7 @@
       </c>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" spans="1:17">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A96" s="28">
         <v>61</v>
       </c>
@@ -10030,7 +10030,7 @@
       </c>
       <c r="Q96" s="42"/>
     </row>
-    <row r="97" spans="1:17">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A97" s="28">
         <v>205</v>
       </c>
@@ -10069,7 +10069,7 @@
       </c>
       <c r="Q97" s="42"/>
     </row>
-    <row r="98" spans="1:17">
+    <row r="98" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A98" s="36">
         <v>62</v>
       </c>
@@ -10100,7 +10100,7 @@
       </c>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" spans="1:17">
+    <row r="99" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A99" s="36">
         <v>63</v>
       </c>
@@ -10139,7 +10139,7 @@
       </c>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" spans="1:17">
+    <row r="100" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A100" s="36"/>
       <c r="B100" s="3"/>
       <c r="C100" s="36">
@@ -10168,7 +10168,7 @@
       </c>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" spans="1:17">
+    <row r="101" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="36"/>
       <c r="B101" s="3"/>
       <c r="C101" s="36">
@@ -10197,7 +10197,7 @@
       </c>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" spans="1:17">
+    <row r="102" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A102" s="36">
         <v>64</v>
       </c>
@@ -10238,7 +10238,7 @@
       </c>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" spans="1:17">
+    <row r="103" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A103" s="36"/>
       <c r="B103" s="3"/>
       <c r="C103" s="36">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" spans="1:17">
+    <row r="104" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A104" s="36">
         <v>65</v>
       </c>
@@ -10310,7 +10310,7 @@
       </c>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" spans="1:17">
+    <row r="105" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A105" s="36"/>
       <c r="B105" s="3"/>
       <c r="C105" s="36">
@@ -10341,7 +10341,7 @@
       </c>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" spans="1:17">
+    <row r="106" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A106" s="36">
         <v>66</v>
       </c>
@@ -10380,7 +10380,7 @@
       </c>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" spans="1:17">
+    <row r="107" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" s="36">
         <v>67</v>
       </c>
@@ -10419,7 +10419,7 @@
       </c>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" spans="1:17">
+    <row r="108" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A108" s="36"/>
       <c r="B108" s="3"/>
       <c r="C108" s="36">
@@ -10448,7 +10448,7 @@
       <c r="P108" s="1"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" spans="1:17">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A109" s="36"/>
       <c r="B109" s="3"/>
       <c r="C109" s="36">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="Q109" s="42"/>
     </row>
-    <row r="110" spans="1:17">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A110" s="28">
         <v>68</v>
       </c>
@@ -10514,7 +10514,7 @@
       </c>
       <c r="Q110" s="42"/>
     </row>
-    <row r="111" spans="1:17">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A111" s="28">
         <v>203</v>
       </c>
@@ -10543,7 +10543,7 @@
       </c>
       <c r="Q111" s="42"/>
     </row>
-    <row r="112" spans="1:17">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A112" s="28">
         <v>51</v>
       </c>
@@ -10582,7 +10582,7 @@
       </c>
       <c r="Q112" s="42"/>
     </row>
-    <row r="113" spans="1:17">
+    <row r="113" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A113" s="28">
         <v>52</v>
       </c>
@@ -10600,7 +10600,7 @@
         <v>377</v>
       </c>
       <c r="G113" s="28">
-        <v>51</v>
+        <v>203</v>
       </c>
       <c r="H113" s="28">
         <v>3</v>
@@ -10621,7 +10621,7 @@
       </c>
       <c r="Q113" s="42"/>
     </row>
-    <row r="114" spans="1:17">
+    <row r="114" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A114" s="28"/>
       <c r="B114" s="21"/>
       <c r="C114" s="28">
@@ -10650,7 +10650,7 @@
       </c>
       <c r="Q114" s="42"/>
     </row>
-    <row r="115" spans="1:17">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A115" s="28"/>
       <c r="B115" s="21"/>
       <c r="C115" s="28">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="Q115" s="42"/>
     </row>
-    <row r="116" spans="1:17">
+    <row r="116" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A116" s="28">
         <v>53</v>
       </c>
@@ -10697,7 +10697,7 @@
         <v>160</v>
       </c>
       <c r="G116" s="28">
-        <v>51</v>
+        <v>203</v>
       </c>
       <c r="H116" s="28">
         <v>3</v>
@@ -10718,7 +10718,7 @@
       </c>
       <c r="Q116" s="35"/>
     </row>
-    <row r="117" spans="1:17">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A117" s="28">
         <v>213</v>
       </c>
@@ -10747,7 +10747,7 @@
       </c>
       <c r="Q117" s="42"/>
     </row>
-    <row r="118" spans="1:17">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A118" s="28">
         <v>69</v>
       </c>
@@ -10784,7 +10784,7 @@
       </c>
       <c r="Q118" s="42"/>
     </row>
-    <row r="119" spans="1:17">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A119" s="28"/>
       <c r="B119" s="21"/>
       <c r="C119" s="28">
@@ -10813,7 +10813,7 @@
       </c>
       <c r="Q119" s="42"/>
     </row>
-    <row r="120" spans="1:17">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A120" s="28"/>
       <c r="B120" s="21"/>
       <c r="C120" s="28">
@@ -10842,7 +10842,7 @@
       </c>
       <c r="Q120" s="42"/>
     </row>
-    <row r="121" spans="1:17">
+    <row r="121" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A121" s="28">
         <v>70</v>
       </c>
@@ -10881,7 +10881,7 @@
       </c>
       <c r="Q121" s="35"/>
     </row>
-    <row r="122" spans="1:17">
+    <row r="122" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A122" s="28"/>
       <c r="B122" s="21"/>
       <c r="C122" s="28">
@@ -10910,7 +10910,7 @@
       </c>
       <c r="Q122" s="35"/>
     </row>
-    <row r="123" spans="1:17">
+    <row r="123" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A123" s="28"/>
       <c r="B123" s="21"/>
       <c r="C123" s="28">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="Q123" s="35"/>
     </row>
-    <row r="124" spans="1:17">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A124" s="36">
         <v>72</v>
       </c>
@@ -10969,7 +10969,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="125" spans="1:17">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A125" s="36">
         <v>73</v>
       </c>
@@ -11005,7 +11005,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="126" spans="1:17">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A126" s="36"/>
       <c r="B126" s="3"/>
       <c r="C126" s="36">
@@ -11033,7 +11033,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="127" spans="1:17">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A127" s="36">
         <v>75</v>
       </c>
@@ -11071,7 +11071,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="128" spans="1:17">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A128" s="36"/>
       <c r="B128" s="3"/>
       <c r="C128" s="36">
@@ -11099,7 +11099,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="129" spans="1:17">
+    <row r="129" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A129" s="36"/>
       <c r="B129" s="3"/>
       <c r="C129" s="36">
@@ -11127,7 +11127,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="130" spans="1:17">
+    <row r="130" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A130" s="36">
         <v>76</v>
       </c>
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="131" spans="1:17">
+    <row r="131" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A131" s="36">
         <v>78</v>
       </c>
@@ -11206,7 +11206,7 @@
       </c>
       <c r="Q131" s="35"/>
     </row>
-    <row r="132" spans="1:17">
+    <row r="132" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A132" s="36"/>
       <c r="B132" s="3"/>
       <c r="C132" s="36">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="Q132" s="35"/>
     </row>
-    <row r="133" spans="1:17">
+    <row r="133" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A133" s="36"/>
       <c r="B133" s="3"/>
       <c r="C133" s="36">
@@ -11264,7 +11264,7 @@
       </c>
       <c r="Q133" s="35"/>
     </row>
-    <row r="134" spans="1:17">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A134" s="36">
         <v>79</v>
       </c>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="Q134" s="42"/>
     </row>
-    <row r="135" spans="1:17">
+    <row r="135" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A135" s="28">
         <v>80</v>
       </c>
@@ -11340,7 +11340,7 @@
       </c>
       <c r="Q135" s="35"/>
     </row>
-    <row r="136" spans="1:17">
+    <row r="136" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A136" s="28">
         <v>81</v>
       </c>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="Q136" s="35"/>
     </row>
-    <row r="137" spans="1:17">
+    <row r="137" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A137" s="28">
         <v>82</v>
       </c>
@@ -11420,7 +11420,7 @@
       </c>
       <c r="Q137" s="35"/>
     </row>
-    <row r="138" spans="1:17">
+    <row r="138" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A138" s="28">
         <v>83</v>
       </c>
@@ -11461,7 +11461,7 @@
       </c>
       <c r="Q138" s="35"/>
     </row>
-    <row r="139" spans="1:17">
+    <row r="139" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A139" s="28"/>
       <c r="B139" s="21"/>
       <c r="C139" s="28">
@@ -11490,7 +11490,7 @@
       </c>
       <c r="Q139" s="35"/>
     </row>
-    <row r="140" spans="1:17">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A140" s="28">
         <v>84</v>
       </c>
@@ -11531,7 +11531,7 @@
       </c>
       <c r="Q140" s="42"/>
     </row>
-    <row r="141" spans="1:17">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A141" s="28"/>
       <c r="B141" s="21"/>
       <c r="C141" s="28">
@@ -11560,7 +11560,7 @@
       </c>
       <c r="Q141" s="42"/>
     </row>
-    <row r="142" spans="1:17">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A142" s="28"/>
       <c r="B142" s="21"/>
       <c r="C142" s="28">
@@ -11589,7 +11589,7 @@
       </c>
       <c r="Q142" s="42"/>
     </row>
-    <row r="143" spans="1:17">
+    <row r="143" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A143" s="36">
         <v>206</v>
       </c>
@@ -11620,7 +11620,7 @@
       </c>
       <c r="Q143" s="35"/>
     </row>
-    <row r="144" spans="1:17">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A144" s="36">
         <v>85</v>
       </c>
@@ -11659,7 +11659,7 @@
       </c>
       <c r="Q144" s="42"/>
     </row>
-    <row r="145" spans="1:17">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A145" s="36"/>
       <c r="B145" s="3"/>
       <c r="C145" s="36">
@@ -11688,7 +11688,7 @@
       </c>
       <c r="Q145" s="42"/>
     </row>
-    <row r="146" spans="1:17">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A146" s="36"/>
       <c r="B146" s="3"/>
       <c r="C146" s="36">
@@ -11717,7 +11717,7 @@
       </c>
       <c r="Q146" s="42"/>
     </row>
-    <row r="147" spans="1:17">
+    <row r="147" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A147" s="36"/>
       <c r="B147" s="3"/>
       <c r="C147" s="36">
@@ -11750,7 +11750,7 @@
       </c>
       <c r="Q147" s="35"/>
     </row>
-    <row r="148" spans="1:17">
+    <row r="148" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A148" s="36">
         <v>86</v>
       </c>
@@ -11791,7 +11791,7 @@
       </c>
       <c r="Q148" s="35"/>
     </row>
-    <row r="149" spans="1:17">
+    <row r="149" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A149" s="36"/>
       <c r="B149" s="3"/>
       <c r="C149" s="36">
@@ -11820,7 +11820,7 @@
       </c>
       <c r="Q149" s="35"/>
     </row>
-    <row r="150" spans="1:17">
+    <row r="150" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A150" s="36">
         <v>87</v>
       </c>
@@ -11861,7 +11861,7 @@
       </c>
       <c r="Q150" s="35"/>
     </row>
-    <row r="151" spans="1:17">
+    <row r="151" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A151" s="36">
         <v>88</v>
       </c>
@@ -11902,7 +11902,7 @@
       </c>
       <c r="Q151" s="35"/>
     </row>
-    <row r="152" spans="1:17">
+    <row r="152" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A152" s="36">
         <v>89</v>
       </c>
@@ -11943,7 +11943,7 @@
       </c>
       <c r="Q152" s="35"/>
     </row>
-    <row r="153" spans="1:17">
+    <row r="153" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A153" s="36">
         <v>90</v>
       </c>
@@ -11984,7 +11984,7 @@
       </c>
       <c r="Q153" s="35"/>
     </row>
-    <row r="154" spans="1:17">
+    <row r="154" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A154" s="36">
         <v>91</v>
       </c>
@@ -12025,7 +12025,7 @@
       </c>
       <c r="Q154" s="35"/>
     </row>
-    <row r="155" spans="1:17">
+    <row r="155" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A155" s="36">
         <v>92</v>
       </c>
@@ -12066,7 +12066,7 @@
       </c>
       <c r="Q155" s="42"/>
     </row>
-    <row r="156" spans="1:17">
+    <row r="156" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A156" s="28">
         <v>93</v>
       </c>
@@ -12101,7 +12101,7 @@
       </c>
       <c r="Q156" s="35"/>
     </row>
-    <row r="157" spans="1:17">
+    <row r="157" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A157" s="28"/>
       <c r="B157" s="21"/>
       <c r="C157" s="28">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="Q157" s="35"/>
     </row>
-    <row r="158" spans="1:17">
+    <row r="158" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A158" s="28">
         <v>94</v>
       </c>
@@ -12167,7 +12167,7 @@
       </c>
       <c r="Q158" s="35"/>
     </row>
-    <row r="159" spans="1:17">
+    <row r="159" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A159" s="28">
         <v>95</v>
       </c>
@@ -12208,7 +12208,7 @@
       </c>
       <c r="Q159" s="35"/>
     </row>
-    <row r="160" spans="1:17">
+    <row r="160" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A160" s="28"/>
       <c r="B160" s="21"/>
       <c r="C160" s="28">
@@ -12235,7 +12235,7 @@
       <c r="P160" s="2"/>
       <c r="Q160" s="35"/>
     </row>
-    <row r="161" spans="1:17">
+    <row r="161" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A161" s="28"/>
       <c r="B161" s="21"/>
       <c r="C161" s="28">
@@ -12264,7 +12264,7 @@
       <c r="P161" s="2"/>
       <c r="Q161" s="35"/>
     </row>
-    <row r="162" spans="1:17">
+    <row r="162" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A162" s="28">
         <v>96</v>
       </c>
@@ -12307,7 +12307,7 @@
       </c>
       <c r="Q162" s="35"/>
     </row>
-    <row r="163" spans="1:17">
+    <row r="163" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A163" s="28">
         <v>97</v>
       </c>
@@ -12350,7 +12350,7 @@
       </c>
       <c r="Q163" s="35"/>
     </row>
-    <row r="164" spans="1:17">
+    <row r="164" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A164" s="28"/>
       <c r="B164" s="21"/>
       <c r="C164" s="28">
@@ -12379,7 +12379,7 @@
       <c r="P164" s="2"/>
       <c r="Q164" s="35"/>
     </row>
-    <row r="165" spans="1:17">
+    <row r="165" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A165" s="36">
         <v>207</v>
       </c>
@@ -12410,7 +12410,7 @@
       </c>
       <c r="Q165" s="35"/>
     </row>
-    <row r="166" spans="1:17">
+    <row r="166" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A166" s="36">
         <v>98</v>
       </c>
@@ -12447,7 +12447,7 @@
       <c r="P166" s="1"/>
       <c r="Q166" s="35"/>
     </row>
-    <row r="167" spans="1:17">
+    <row r="167" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A167" s="36">
         <v>99</v>
       </c>
@@ -12487,7 +12487,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="168" spans="1:17">
+    <row r="168" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A168" s="36"/>
       <c r="B168" s="3"/>
       <c r="C168" s="36">
@@ -12515,7 +12515,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="169" spans="1:17">
+    <row r="169" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A169" s="28">
         <v>100</v>
       </c>
@@ -12546,7 +12546,7 @@
       </c>
       <c r="Q169" s="35"/>
     </row>
-    <row r="170" spans="1:17">
+    <row r="170" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A170" s="28">
         <v>101</v>
       </c>
@@ -12585,7 +12585,7 @@
       </c>
       <c r="Q170" s="35"/>
     </row>
-    <row r="171" spans="1:17">
+    <row r="171" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A171" s="28"/>
       <c r="B171" s="21"/>
       <c r="C171" s="28">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="Q171" s="35"/>
     </row>
-    <row r="172" spans="1:17">
+    <row r="172" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A172" s="28">
         <v>102</v>
       </c>
@@ -12655,7 +12655,7 @@
       </c>
       <c r="Q172" s="35"/>
     </row>
-    <row r="173" spans="1:17">
+    <row r="173" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A173" s="28"/>
       <c r="B173" s="21"/>
       <c r="C173" s="28">
@@ -12686,7 +12686,7 @@
       </c>
       <c r="Q173" s="42"/>
     </row>
-    <row r="174" spans="1:17">
+    <row r="174" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A174" s="36">
         <v>103</v>
       </c>
@@ -12717,7 +12717,7 @@
       </c>
       <c r="Q174" s="35"/>
     </row>
-    <row r="175" spans="1:17">
+    <row r="175" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A175" s="28">
         <v>71</v>
       </c>
@@ -12755,7 +12755,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="176" spans="1:17">
+    <row r="176" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A176" s="36">
         <v>104</v>
       </c>
@@ -12796,7 +12796,7 @@
       </c>
       <c r="Q176" s="35"/>
     </row>
-    <row r="177" spans="1:17">
+    <row r="177" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A177" s="36">
         <v>105</v>
       </c>
@@ -12839,7 +12839,7 @@
       </c>
       <c r="Q177" s="35"/>
     </row>
-    <row r="178" spans="1:17">
+    <row r="178" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A178" s="36">
         <v>106</v>
       </c>
@@ -12881,7 +12881,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="179" spans="1:17">
+    <row r="179" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A179" s="28">
         <v>107</v>
       </c>
@@ -12919,7 +12919,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="180" spans="1:17">
+    <row r="180" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A180" s="28"/>
       <c r="B180" s="21"/>
       <c r="C180" s="28">
@@ -12947,7 +12947,7 @@
       <c r="O180" s="2"/>
       <c r="P180" s="2"/>
     </row>
-    <row r="181" spans="1:17">
+    <row r="181" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A181" s="28"/>
       <c r="B181" s="21"/>
       <c r="C181" s="28">
@@ -12975,7 +12975,7 @@
       <c r="O181" s="2"/>
       <c r="P181" s="2"/>
     </row>
-    <row r="182" spans="1:17">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A182" s="36">
         <v>209</v>
       </c>
@@ -13005,7 +13005,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="183" spans="1:17">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A183" s="36">
         <v>108</v>
       </c>
@@ -13039,7 +13039,7 @@
       <c r="O183" s="1"/>
       <c r="P183" s="1"/>
     </row>
-    <row r="184" spans="1:17">
+    <row r="184" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A184" s="36">
         <v>109</v>
       </c>
@@ -13077,11 +13077,11 @@
         <v>569</v>
       </c>
     </row>
-    <row r="185" spans="1:17">
+    <row r="185" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A185" s="61"/>
       <c r="C185" s="61"/>
     </row>
-    <row r="186" spans="1:17">
+    <row r="186" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A186" s="61"/>
       <c r="C186" s="61"/>
     </row>
@@ -13092,23 +13092,23 @@
   <conditionalFormatting sqref="C1:C1048576">
     <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J161:J1048576 J1:J159">
+    <cfRule type="duplicateValues" dxfId="7" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K161:K1048576 K1:K159">
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="16"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L1:L1048576">
-    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:M1048576">
-    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:N1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J161:J1048576 J1:J159">
-    <cfRule type="duplicateValues" dxfId="2" priority="13"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K161:K1048576 K1:K159">
-    <cfRule type="duplicateValues" dxfId="1" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.70069444444444395" right="0.70069444444444395" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13118,26 +13118,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="4" width="7.140625" customWidth="1"/>
+    <col min="1" max="2" width="35.6640625" customWidth="1"/>
+    <col min="3" max="4" width="7.1640625" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
-    <col min="6" max="8" width="28.42578125" customWidth="1"/>
-    <col min="10" max="10" width="42.85546875" customWidth="1"/>
+    <col min="6" max="8" width="28.5" customWidth="1"/>
+    <col min="10" max="10" width="42.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="95" t="s">
         <v>2</v>
       </c>
@@ -13162,7 +13162,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="45">
+    <row r="5" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="96"/>
       <c r="B5" s="96"/>
       <c r="C5" s="1" t="s">
@@ -13179,7 +13179,7 @@
       </c>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" ht="45">
+    <row r="6" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="21"/>
       <c r="B6" s="21"/>
       <c r="C6" s="2"/>
@@ -13198,7 +13198,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="60">
+    <row r="7" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A7" s="21"/>
       <c r="B7" s="21"/>
       <c r="C7" s="2"/>
@@ -13215,7 +13215,7 @@
       </c>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" ht="60">
+    <row r="8" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A8" s="21"/>
       <c r="B8" s="21"/>
       <c r="C8" s="2"/>
@@ -13232,7 +13232,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="30">
+    <row r="9" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="21"/>
       <c r="B9" s="21"/>
       <c r="C9" s="2"/>
@@ -13249,7 +13249,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="30">
+    <row r="10" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="21"/>
       <c r="B10" s="21"/>
       <c r="C10" s="2"/>
@@ -13268,7 +13268,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30">
+    <row r="11" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="21"/>
       <c r="B11" s="21"/>
       <c r="C11" s="2"/>
@@ -13287,7 +13287,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="30">
+    <row r="12" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="21"/>
       <c r="B12" s="21"/>
       <c r="C12" s="2"/>
@@ -13304,7 +13304,7 @@
       </c>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10" ht="30">
+    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="21"/>
       <c r="B13" s="21"/>
       <c r="C13" s="2"/>
@@ -13321,7 +13321,7 @@
       </c>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10" ht="30">
+    <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="21"/>
       <c r="B14" s="21"/>
       <c r="C14" s="2"/>
@@ -13338,7 +13338,7 @@
       </c>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" ht="30">
+    <row r="15" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="21"/>
       <c r="B15" s="21"/>
       <c r="C15" s="2"/>
@@ -13355,7 +13355,7 @@
       </c>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10" ht="60">
+    <row r="16" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A16" s="21"/>
       <c r="B16" s="21"/>
       <c r="C16" s="2"/>
@@ -13368,7 +13368,7 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="1:10" ht="75">
+    <row r="17" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A17" s="21"/>
       <c r="B17" s="21"/>
       <c r="C17" s="2"/>
@@ -13381,11 +13381,11 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="62"/>
       <c r="B18" s="62"/>
     </row>
-    <row r="19" spans="1:10" ht="45">
+    <row r="19" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>77</v>
       </c>

</xml_diff>

<commit_message>
updated Kompetenzraster and mcqs
- MCQ SC score = 1
- MCQ MC score = 0.5/option
</commit_message>
<xml_diff>
--- a/files/Kompetenzraster.xlsx
+++ b/files/Kompetenzraster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcsauer/GitHub/hefl/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A937983-5877-41CD-B8D2-B6E9DA066118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B615E0CC-F4DC-7146-8A27-1B5B8737AAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OFP" sheetId="1" r:id="rId1"/>
@@ -1907,9 +1907,6 @@
     <t>2,17,210</t>
   </si>
   <si>
-    <t>2,10,11,12,13,15,210</t>
-  </si>
-  <si>
     <t>2,18,201</t>
   </si>
   <si>
@@ -2040,13 +2037,16 @@
   </si>
   <si>
     <t>mehrdimensionales Array</t>
+  </si>
+  <si>
+    <t>2,15,210</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2661,9 +2661,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2701,7 +2701,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2807,7 +2807,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2949,7 +2949,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2958,25 +2958,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I245"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="4" width="7.140625" customWidth="1"/>
+    <col min="1" max="2" width="35.6640625" customWidth="1"/>
+    <col min="3" max="4" width="7.1640625" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
-    <col min="6" max="9" width="28.42578125" customWidth="1"/>
+    <col min="6" max="9" width="28.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="96" t="s">
         <v>2</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30">
+    <row r="5" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="97" t="s">
         <v>7</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="30">
+    <row r="6" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="94" t="s">
         <v>12</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="30">
+    <row r="7" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="95" t="s">
         <v>17</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="60">
+    <row r="8" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="94" t="s">
         <v>22</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="45">
+    <row r="9" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="45">
+    <row r="10" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="7"/>
       <c r="B10" s="7" t="s">
         <v>32</v>
@@ -3124,7 +3124,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="45">
+    <row r="11" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="7"/>
       <c r="B11" s="7" t="s">
         <v>36</v>
@@ -3146,7 +3146,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="30">
+    <row r="12" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="7"/>
       <c r="B12" s="7" t="s">
         <v>42</v>
@@ -3168,7 +3168,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="75">
+    <row r="13" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="B13" s="7" t="s">
         <v>46</v>
@@ -3190,7 +3190,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="60">
+    <row r="14" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A14" s="7"/>
       <c r="B14" s="7" t="s">
         <v>50</v>
@@ -3210,7 +3210,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="94" t="s">
         <v>55</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="45">
+    <row r="16" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A16" s="95" t="s">
         <v>60</v>
       </c>
@@ -3250,7 +3250,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60">
+    <row r="17" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>65</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="2" t="s">
         <v>67</v>
@@ -3268,7 +3268,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="2" t="s">
         <v>69</v>
@@ -3277,7 +3277,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="2" t="s">
         <v>71</v>
@@ -3286,7 +3286,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="2" t="s">
         <v>73</v>
@@ -3295,7 +3295,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="2" t="s">
         <v>75</v>
@@ -3304,7 +3304,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="45">
+    <row r="24" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>77</v>
       </c>
@@ -3330,7 +3330,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>67</v>
       </c>
@@ -3342,7 +3342,7 @@
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
     </row>
-    <row r="26" spans="1:8" s="13" customFormat="1">
+    <row r="26" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>85</v>
       </c>
@@ -3358,7 +3358,7 @@
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
     </row>
-    <row r="27" spans="1:8" s="13" customFormat="1">
+    <row r="27" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
         <v>88</v>
@@ -3372,7 +3372,7 @@
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
     </row>
-    <row r="28" spans="1:8" s="13" customFormat="1">
+    <row r="28" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="11"/>
@@ -3384,7 +3384,7 @@
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>90</v>
       </c>
@@ -3398,7 +3398,7 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>85</v>
       </c>
@@ -3412,7 +3412,7 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
         <v>91</v>
@@ -3426,7 +3426,7 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="7"/>
@@ -3438,7 +3438,7 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>92</v>
       </c>
@@ -3450,7 +3450,7 @@
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" s="13" customFormat="1">
+    <row r="34" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>85</v>
       </c>
@@ -3466,7 +3466,7 @@
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="1:8" s="13" customFormat="1">
+    <row r="35" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="17"/>
       <c r="C35" s="2"/>
@@ -3478,7 +3478,7 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="1:8" s="13" customFormat="1">
+    <row r="36" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="17" t="s">
         <v>94</v>
@@ -3490,7 +3490,7 @@
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" s="13" customFormat="1">
+    <row r="37" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2" t="s">
         <v>95</v>
@@ -3504,7 +3504,7 @@
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="1:8" s="13" customFormat="1">
+    <row r="38" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -3516,7 +3516,7 @@
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="1:8" s="13" customFormat="1">
+    <row r="39" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2" t="s">
         <v>96</v>
@@ -3530,7 +3530,7 @@
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="1:8" s="13" customFormat="1">
+    <row r="40" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -3542,7 +3542,7 @@
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="1:8" s="13" customFormat="1">
+    <row r="41" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2" t="s">
         <v>97</v>
@@ -3556,7 +3556,7 @@
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="1:8" s="13" customFormat="1">
+    <row r="42" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -3568,7 +3568,7 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" s="13" customFormat="1">
+    <row r="43" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2" t="s">
         <v>98</v>
@@ -3582,7 +3582,7 @@
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="1:8" s="13" customFormat="1">
+    <row r="44" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -3594,7 +3594,7 @@
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="1:8" s="13" customFormat="1">
+    <row r="45" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="2" t="s">
         <v>99</v>
@@ -3608,7 +3608,7 @@
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="1:8" s="13" customFormat="1">
+    <row r="46" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -3620,7 +3620,7 @@
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="1:8" s="13" customFormat="1">
+    <row r="47" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="2" t="s">
         <v>100</v>
@@ -3634,7 +3634,7 @@
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="1:8" s="13" customFormat="1">
+    <row r="48" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -3646,7 +3646,7 @@
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="1:8" s="13" customFormat="1">
+    <row r="49" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2" t="s">
         <v>101</v>
@@ -3660,7 +3660,7 @@
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="1:8" s="13" customFormat="1">
+    <row r="50" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -3672,7 +3672,7 @@
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="1:8" s="13" customFormat="1">
+    <row r="51" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>102</v>
       </c>
@@ -3684,7 +3684,7 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
     </row>
-    <row r="52" spans="1:8" s="13" customFormat="1">
+    <row r="52" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>85</v>
       </c>
@@ -3698,7 +3698,7 @@
       <c r="G52" s="14"/>
       <c r="H52" s="14"/>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="1"/>
       <c r="B53" s="1" t="s">
         <v>103</v>
@@ -3712,7 +3712,7 @@
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -3724,7 +3724,7 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="1"/>
       <c r="B55" s="1" t="s">
         <v>105</v>
@@ -3736,7 +3736,7 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="1"/>
       <c r="B56" s="1" t="s">
         <v>106</v>
@@ -3750,7 +3750,7 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -3762,7 +3762,7 @@
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="1"/>
       <c r="B58" s="1" t="s">
         <v>107</v>
@@ -3776,7 +3776,7 @@
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -3788,7 +3788,7 @@
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -3800,7 +3800,7 @@
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>108</v>
       </c>
@@ -3814,7 +3814,7 @@
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>85</v>
       </c>
@@ -3828,7 +3828,7 @@
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -3840,7 +3840,7 @@
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -3852,7 +3852,7 @@
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2" t="s">
         <v>109</v>
@@ -3866,7 +3866,7 @@
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="2" t="s">
         <v>110</v>
@@ -3880,7 +3880,7 @@
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -3892,7 +3892,7 @@
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="2" t="s">
         <v>111</v>
@@ -3906,7 +3906,7 @@
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -3918,7 +3918,7 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="2" t="s">
         <v>112</v>
@@ -3932,7 +3932,7 @@
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -3944,7 +3944,7 @@
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -3956,7 +3956,7 @@
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2" t="s">
         <v>113</v>
@@ -3970,7 +3970,7 @@
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="2" t="s">
         <v>114</v>
@@ -3984,7 +3984,7 @@
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -3996,7 +3996,7 @@
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="2" t="s">
         <v>73</v>
@@ -4010,7 +4010,7 @@
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -4022,7 +4022,7 @@
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="1:8" ht="30">
+    <row r="78" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>115</v>
       </c>
@@ -4038,7 +4038,7 @@
       <c r="G78" s="1"/>
       <c r="H78" s="1"/>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
         <v>85</v>
       </c>
@@ -4052,7 +4052,7 @@
       <c r="G79" s="1"/>
       <c r="H79" s="1"/>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
         <v>85</v>
       </c>
@@ -4068,7 +4068,7 @@
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="7"/>
       <c r="B81" s="7"/>
       <c r="C81" s="1"/>
@@ -4080,7 +4080,7 @@
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="8" t="s">
         <v>60</v>
       </c>
@@ -4092,7 +4092,7 @@
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2" t="s">
         <v>118</v>
@@ -4106,7 +4106,7 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -4118,7 +4118,7 @@
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>85</v>
       </c>
@@ -4134,7 +4134,7 @@
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="1:8">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -4146,7 +4146,7 @@
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -4158,7 +4158,7 @@
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="2" t="s">
         <v>119</v>
@@ -4174,7 +4174,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>121</v>
       </c>
@@ -4188,7 +4188,7 @@
       <c r="G89" s="1"/>
       <c r="H89" s="1"/>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>85</v>
       </c>
@@ -4202,7 +4202,7 @@
       <c r="G90" s="1"/>
       <c r="H90" s="1"/>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -4214,7 +4214,7 @@
       <c r="G91" s="1"/>
       <c r="H91" s="1"/>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -4226,7 +4226,7 @@
       <c r="G92" s="1"/>
       <c r="H92" s="1"/>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -4238,7 +4238,7 @@
       <c r="G93" s="1"/>
       <c r="H93" s="1"/>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -4250,7 +4250,7 @@
       <c r="G94" s="1"/>
       <c r="H94" s="1"/>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" s="1"/>
       <c r="B95" s="1" t="s">
         <v>109</v>
@@ -4264,7 +4264,7 @@
       <c r="G95" s="1"/>
       <c r="H95" s="1"/>
     </row>
-    <row r="96" spans="1:8">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -4276,7 +4276,7 @@
       <c r="G96" s="1"/>
       <c r="H96" s="1"/>
     </row>
-    <row r="97" spans="1:8">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>122</v>
       </c>
@@ -4288,7 +4288,7 @@
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="1:8">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="2" t="s">
         <v>123</v>
@@ -4302,7 +4302,7 @@
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="1:8">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -4314,7 +4314,7 @@
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="1:8">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -4326,7 +4326,7 @@
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="1:8">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101" s="2"/>
       <c r="B101" s="2" t="s">
         <v>124</v>
@@ -4340,7 +4340,7 @@
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="1:8">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -4352,7 +4352,7 @@
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="1:8">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -4364,7 +4364,7 @@
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="1:8">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -4376,7 +4376,7 @@
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="1:8">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" s="2"/>
       <c r="B105" s="2" t="s">
         <v>125</v>
@@ -4390,7 +4390,7 @@
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="1:8">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -4402,7 +4402,7 @@
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="1:8">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -4414,7 +4414,7 @@
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="1:8">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>126</v>
       </c>
@@ -4426,7 +4426,7 @@
       <c r="G108" s="1"/>
       <c r="H108" s="1"/>
     </row>
-    <row r="109" spans="1:8">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>85</v>
       </c>
@@ -4442,7 +4442,7 @@
       <c r="G109" s="1"/>
       <c r="H109" s="1"/>
     </row>
-    <row r="110" spans="1:8">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -4454,7 +4454,7 @@
       <c r="G110" s="1"/>
       <c r="H110" s="1"/>
     </row>
-    <row r="111" spans="1:8">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A111" s="1"/>
       <c r="B111" s="1" t="s">
         <v>128</v>
@@ -4468,7 +4468,7 @@
       <c r="G111" s="1"/>
       <c r="H111" s="1"/>
     </row>
-    <row r="112" spans="1:8">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A112" s="1"/>
       <c r="B112" s="1" t="s">
         <v>129</v>
@@ -4482,7 +4482,7 @@
       <c r="G112" s="1"/>
       <c r="H112" s="1"/>
     </row>
-    <row r="114" spans="1:8" ht="30">
+    <row r="114" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A114" s="19" t="s">
         <v>130</v>
       </c>
@@ -4496,7 +4496,7 @@
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="1:8">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
         <v>131</v>
       </c>
@@ -4510,7 +4510,7 @@
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A116" s="3" t="s">
         <v>132</v>
       </c>
@@ -4524,7 +4524,7 @@
       <c r="G116" s="1"/>
       <c r="H116" s="1"/>
     </row>
-    <row r="117" spans="1:8">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>131</v>
       </c>
@@ -4538,7 +4538,7 @@
       <c r="G117" s="1"/>
       <c r="H117" s="1"/>
     </row>
-    <row r="118" spans="1:8">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
         <v>92</v>
       </c>
@@ -4552,7 +4552,7 @@
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="1:8">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -4564,7 +4564,7 @@
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="1:8">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
         <v>131</v>
       </c>
@@ -4580,7 +4580,7 @@
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="1:8">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -4592,7 +4592,7 @@
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="1:8">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A122" s="2"/>
       <c r="B122" s="2" t="s">
         <v>134</v>
@@ -4606,7 +4606,7 @@
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="1:8">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -4618,7 +4618,7 @@
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="1:8">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A124" s="2"/>
       <c r="B124" s="2" t="s">
         <v>135</v>
@@ -4632,7 +4632,7 @@
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="1:8">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -4644,7 +4644,7 @@
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="1:8">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A126" s="2"/>
       <c r="B126" s="2" t="s">
         <v>97</v>
@@ -4658,7 +4658,7 @@
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="1:8">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -4670,7 +4670,7 @@
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="1:8">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A128" s="2"/>
       <c r="B128" s="2" t="s">
         <v>93</v>
@@ -4684,7 +4684,7 @@
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="1:8">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -4696,7 +4696,7 @@
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="1:8">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -4708,7 +4708,7 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="1:8">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A131" s="2"/>
       <c r="B131" s="2" t="s">
         <v>136</v>
@@ -4722,7 +4722,7 @@
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="1:8">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -4734,7 +4734,7 @@
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="1:8">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A133" s="2"/>
       <c r="B133" s="2" t="s">
         <v>137</v>
@@ -4748,7 +4748,7 @@
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="1:8">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -4760,7 +4760,7 @@
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="1:8">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A135" s="2"/>
       <c r="B135" s="2" t="s">
         <v>138</v>
@@ -4774,7 +4774,7 @@
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="1:8">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -4786,7 +4786,7 @@
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="1:8">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A137" s="2"/>
       <c r="B137" s="2" t="s">
         <v>139</v>
@@ -4800,7 +4800,7 @@
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="1:8">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -4812,7 +4812,7 @@
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="1:8">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>90</v>
       </c>
@@ -4826,7 +4826,7 @@
       <c r="G139" s="1"/>
       <c r="H139" s="1"/>
     </row>
-    <row r="140" spans="1:8">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>131</v>
       </c>
@@ -4840,7 +4840,7 @@
       <c r="G140" s="1"/>
       <c r="H140" s="1"/>
     </row>
-    <row r="141" spans="1:8">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
         <v>140</v>
       </c>
@@ -4852,7 +4852,7 @@
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="1:8">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
         <v>131</v>
       </c>
@@ -4868,7 +4868,7 @@
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="1:8">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
@@ -4880,7 +4880,7 @@
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="1:8">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A144" s="2"/>
       <c r="B144" s="2" t="s">
         <v>142</v>
@@ -4894,7 +4894,7 @@
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="1:8">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -4906,7 +4906,7 @@
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="1:8">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A146" s="2"/>
       <c r="B146" s="2" t="s">
         <v>143</v>
@@ -4920,7 +4920,7 @@
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="1:8">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -4932,7 +4932,7 @@
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="1:8">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A148" s="2"/>
       <c r="B148" s="2" t="s">
         <v>144</v>
@@ -4946,7 +4946,7 @@
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="1:8">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -4958,7 +4958,7 @@
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="1:8">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A150" s="2"/>
       <c r="B150" s="2" t="s">
         <v>145</v>
@@ -4972,7 +4972,7 @@
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="1:8">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -4984,7 +4984,7 @@
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="1:8">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>146</v>
       </c>
@@ -4996,7 +4996,7 @@
       <c r="G152" s="1"/>
       <c r="H152" s="1"/>
     </row>
-    <row r="153" spans="1:8">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>131</v>
       </c>
@@ -5012,7 +5012,7 @@
       <c r="G153" s="1"/>
       <c r="H153" s="1"/>
     </row>
-    <row r="154" spans="1:8">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -5024,7 +5024,7 @@
       <c r="G154" s="1"/>
       <c r="H154" s="1"/>
     </row>
-    <row r="155" spans="1:8">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A155" s="1"/>
       <c r="B155" s="1" t="s">
         <v>147</v>
@@ -5038,7 +5038,7 @@
       <c r="G155" s="1"/>
       <c r="H155" s="1"/>
     </row>
-    <row r="156" spans="1:8">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -5050,7 +5050,7 @@
       <c r="G156" s="1"/>
       <c r="H156" s="1"/>
     </row>
-    <row r="157" spans="1:8">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A157" s="1"/>
       <c r="B157" s="1" t="s">
         <v>105</v>
@@ -5064,7 +5064,7 @@
       <c r="G157" s="1"/>
       <c r="H157" s="1"/>
     </row>
-    <row r="158" spans="1:8">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -5076,7 +5076,7 @@
       <c r="G158" s="1"/>
       <c r="H158" s="1"/>
     </row>
-    <row r="159" spans="1:8">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A159" s="1"/>
       <c r="B159" s="1" t="s">
         <v>106</v>
@@ -5090,7 +5090,7 @@
       <c r="G159" s="1"/>
       <c r="H159" s="1"/>
     </row>
-    <row r="160" spans="1:8">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -5102,7 +5102,7 @@
       <c r="G160" s="1"/>
       <c r="H160" s="1"/>
     </row>
-    <row r="161" spans="1:8">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A161" s="1"/>
       <c r="B161" s="1" t="s">
         <v>148</v>
@@ -5116,7 +5116,7 @@
       <c r="G161" s="1"/>
       <c r="H161" s="1"/>
     </row>
-    <row r="162" spans="1:8">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -5128,7 +5128,7 @@
       <c r="G162" s="1"/>
       <c r="H162" s="1"/>
     </row>
-    <row r="163" spans="1:8">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A163" s="1"/>
       <c r="B163" s="1" t="s">
         <v>149</v>
@@ -5142,7 +5142,7 @@
       <c r="G163" s="1"/>
       <c r="H163" s="1"/>
     </row>
-    <row r="164" spans="1:8">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -5154,7 +5154,7 @@
       <c r="G164" s="1"/>
       <c r="H164" s="1"/>
     </row>
-    <row r="165" spans="1:8">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A165" s="17" t="s">
         <v>126</v>
       </c>
@@ -5166,7 +5166,7 @@
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="1:8">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
         <v>131</v>
       </c>
@@ -5182,7 +5182,7 @@
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="1:8">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A167" s="17"/>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
@@ -5194,7 +5194,7 @@
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="1:8">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A168" s="2"/>
       <c r="B168" s="2" t="s">
         <v>151</v>
@@ -5208,7 +5208,7 @@
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="1:8">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
@@ -5220,7 +5220,7 @@
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="1:8">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A170" s="2"/>
       <c r="B170" s="2" t="s">
         <v>152</v>
@@ -5234,7 +5234,7 @@
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="1:8">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
@@ -5246,7 +5246,7 @@
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="1:8">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
         <v>153</v>
       </c>
@@ -5258,7 +5258,7 @@
       <c r="G172" s="1"/>
       <c r="H172" s="1"/>
     </row>
-    <row r="173" spans="1:8">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
         <v>131</v>
       </c>
@@ -5274,7 +5274,7 @@
       <c r="G173" s="1"/>
       <c r="H173" s="1"/>
     </row>
-    <row r="174" spans="1:8">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -5286,7 +5286,7 @@
       <c r="G174" s="1"/>
       <c r="H174" s="1"/>
     </row>
-    <row r="175" spans="1:8">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A175" s="1"/>
       <c r="B175" s="1" t="s">
         <v>155</v>
@@ -5300,7 +5300,7 @@
       <c r="G175" s="1"/>
       <c r="H175" s="1"/>
     </row>
-    <row r="176" spans="1:8">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
@@ -5312,7 +5312,7 @@
       <c r="G176" s="1"/>
       <c r="H176" s="1"/>
     </row>
-    <row r="177" spans="1:8">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A177" s="1"/>
       <c r="B177" s="1" t="s">
         <v>156</v>
@@ -5326,7 +5326,7 @@
       <c r="G177" s="1"/>
       <c r="H177" s="1"/>
     </row>
-    <row r="178" spans="1:8">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
@@ -5338,7 +5338,7 @@
       <c r="G178" s="1"/>
       <c r="H178" s="1"/>
     </row>
-    <row r="179" spans="1:8">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A179" s="1"/>
       <c r="B179" s="1" t="s">
         <v>157</v>
@@ -5352,7 +5352,7 @@
       <c r="G179" s="1"/>
       <c r="H179" s="1"/>
     </row>
-    <row r="180" spans="1:8">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
@@ -5364,7 +5364,7 @@
       <c r="G180" s="1"/>
       <c r="H180" s="1"/>
     </row>
-    <row r="181" spans="1:8">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A181" s="1"/>
       <c r="B181" s="1" t="s">
         <v>158</v>
@@ -5378,7 +5378,7 @@
       <c r="G181" s="1"/>
       <c r="H181" s="1"/>
     </row>
-    <row r="182" spans="1:8">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
@@ -5390,7 +5390,7 @@
       <c r="G182" s="1"/>
       <c r="H182" s="1"/>
     </row>
-    <row r="183" spans="1:8">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A183" s="1"/>
       <c r="B183" s="1" t="s">
         <v>159</v>
@@ -5404,7 +5404,7 @@
       <c r="G183" s="1"/>
       <c r="H183" s="1"/>
     </row>
-    <row r="184" spans="1:8">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
@@ -5416,7 +5416,7 @@
       <c r="G184" s="1"/>
       <c r="H184" s="1"/>
     </row>
-    <row r="185" spans="1:8">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
@@ -5428,7 +5428,7 @@
       <c r="G185" s="1"/>
       <c r="H185" s="1"/>
     </row>
-    <row r="186" spans="1:8">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
         <v>160</v>
       </c>
@@ -5444,7 +5444,7 @@
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="1:8">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
         <v>131</v>
       </c>
@@ -5458,7 +5458,7 @@
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="1:8">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A188" s="2"/>
       <c r="B188" s="2" t="s">
         <v>162</v>
@@ -5472,7 +5472,7 @@
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="1:8">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
@@ -5484,7 +5484,7 @@
       <c r="G189" s="2"/>
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="1:8">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A190" s="2"/>
       <c r="B190" s="2" t="s">
         <v>163</v>
@@ -5498,7 +5498,7 @@
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="1:8">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
@@ -5510,7 +5510,7 @@
       <c r="G191" s="2"/>
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="1:8">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A192" s="2"/>
       <c r="B192" s="2" t="s">
         <v>121</v>
@@ -5524,7 +5524,7 @@
       <c r="G192" s="2"/>
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="1:8">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="2"/>
@@ -5536,7 +5536,7 @@
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="1:8">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
         <v>164</v>
       </c>
@@ -5552,7 +5552,7 @@
       <c r="G194" s="1"/>
       <c r="H194" s="1"/>
     </row>
-    <row r="195" spans="1:8">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
@@ -5564,7 +5564,7 @@
       <c r="G195" s="1"/>
       <c r="H195" s="1"/>
     </row>
-    <row r="196" spans="1:8">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A196" s="1"/>
       <c r="B196" s="1" t="s">
         <v>165</v>
@@ -5578,7 +5578,7 @@
       <c r="G196" s="1"/>
       <c r="H196" s="1"/>
     </row>
-    <row r="197" spans="1:8">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
@@ -5590,7 +5590,7 @@
       <c r="G197" s="1"/>
       <c r="H197" s="1"/>
     </row>
-    <row r="198" spans="1:8">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A198" s="1"/>
       <c r="B198" s="1" t="s">
         <v>155</v>
@@ -5604,7 +5604,7 @@
       <c r="G198" s="1"/>
       <c r="H198" s="1"/>
     </row>
-    <row r="199" spans="1:8">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
@@ -5616,7 +5616,7 @@
       <c r="G199" s="1"/>
       <c r="H199" s="1"/>
     </row>
-    <row r="200" spans="1:8">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A200" s="1"/>
       <c r="B200" s="1" t="s">
         <v>153</v>
@@ -5630,7 +5630,7 @@
       <c r="G200" s="1"/>
       <c r="H200" s="1"/>
     </row>
-    <row r="201" spans="1:8">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
@@ -5642,7 +5642,7 @@
       <c r="G201" s="1"/>
       <c r="H201" s="1"/>
     </row>
-    <row r="202" spans="1:8">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A202" s="1"/>
       <c r="B202" s="1" t="s">
         <v>166</v>
@@ -5656,7 +5656,7 @@
       <c r="G202" s="1"/>
       <c r="H202" s="1"/>
     </row>
-    <row r="203" spans="1:8">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
@@ -5668,7 +5668,7 @@
       <c r="G203" s="1"/>
       <c r="H203" s="1"/>
     </row>
-    <row r="204" spans="1:8">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A204" s="1"/>
       <c r="B204" s="1" t="s">
         <v>167</v>
@@ -5682,7 +5682,7 @@
       <c r="G204" s="1"/>
       <c r="H204" s="1"/>
     </row>
-    <row r="205" spans="1:8">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
@@ -5694,7 +5694,7 @@
       <c r="G205" s="1"/>
       <c r="H205" s="1"/>
     </row>
-    <row r="206" spans="1:8">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A206" s="1"/>
       <c r="B206" s="1" t="s">
         <v>168</v>
@@ -5708,7 +5708,7 @@
       <c r="G206" s="1"/>
       <c r="H206" s="1"/>
     </row>
-    <row r="207" spans="1:8">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
@@ -5720,7 +5720,7 @@
       <c r="G207" s="1"/>
       <c r="H207" s="1"/>
     </row>
-    <row r="208" spans="1:8">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A208" s="1"/>
       <c r="B208" s="1" t="s">
         <v>169</v>
@@ -5734,7 +5734,7 @@
       <c r="G208" s="1"/>
       <c r="H208" s="1"/>
     </row>
-    <row r="209" spans="1:8">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
@@ -5746,7 +5746,7 @@
       <c r="G209" s="1"/>
       <c r="H209" s="1"/>
     </row>
-    <row r="210" spans="1:8">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A210" s="1"/>
       <c r="B210" s="1" t="s">
         <v>170</v>
@@ -5760,7 +5760,7 @@
       <c r="G210" s="1"/>
       <c r="H210" s="1"/>
     </row>
-    <row r="211" spans="1:8">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
@@ -5772,7 +5772,7 @@
       <c r="G211" s="1"/>
       <c r="H211" s="1"/>
     </row>
-    <row r="212" spans="1:8">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A212" s="2" t="s">
         <v>171</v>
       </c>
@@ -5788,7 +5788,7 @@
       <c r="G212" s="2"/>
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="1:8">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
       <c r="C213" s="2"/>
@@ -5800,7 +5800,7 @@
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="1:8">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A214" s="2" t="s">
         <v>131</v>
       </c>
@@ -5816,7 +5816,7 @@
       <c r="G214" s="2"/>
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="1:8">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A215" s="2"/>
       <c r="B215" s="2"/>
       <c r="C215" s="2"/>
@@ -5828,7 +5828,7 @@
       <c r="G215" s="2"/>
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="1:8">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A216" s="2" t="s">
         <v>164</v>
       </c>
@@ -5844,7 +5844,7 @@
       <c r="G216" s="2"/>
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="1:8">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A217" s="2"/>
       <c r="B217" s="2"/>
       <c r="C217" s="2"/>
@@ -5856,7 +5856,7 @@
       <c r="G217" s="2"/>
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="1:8">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A218" s="2"/>
       <c r="B218" s="2"/>
       <c r="C218" s="2"/>
@@ -5868,7 +5868,7 @@
       <c r="G218" s="2"/>
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="1:8">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A219" s="2"/>
       <c r="B219" s="2" t="s">
         <v>171</v>
@@ -5882,7 +5882,7 @@
       <c r="G219" s="2"/>
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="1:8">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A220" s="2"/>
       <c r="B220" s="2"/>
       <c r="C220" s="2"/>
@@ -5894,7 +5894,7 @@
       <c r="G220" s="2"/>
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="1:8">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A221" s="2"/>
       <c r="B221" s="2"/>
       <c r="C221" s="2"/>
@@ -5906,7 +5906,7 @@
       <c r="G221" s="2"/>
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="1:8">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A222" s="1" t="s">
         <v>175</v>
       </c>
@@ -5920,7 +5920,7 @@
       <c r="G222" s="1"/>
       <c r="H222" s="1"/>
     </row>
-    <row r="223" spans="1:8">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="s">
         <v>131</v>
       </c>
@@ -5934,7 +5934,7 @@
       <c r="G223" s="1"/>
       <c r="H223" s="1"/>
     </row>
-    <row r="224" spans="1:8">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A224" s="1"/>
       <c r="B224" s="1" t="s">
         <v>176</v>
@@ -5948,7 +5948,7 @@
       <c r="G224" s="1"/>
       <c r="H224" s="1"/>
     </row>
-    <row r="225" spans="1:8">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A225" s="1"/>
       <c r="B225" s="1"/>
       <c r="C225" s="1"/>
@@ -5960,7 +5960,7 @@
       <c r="G225" s="1"/>
       <c r="H225" s="1"/>
     </row>
-    <row r="226" spans="1:8">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A226" s="2" t="s">
         <v>177</v>
       </c>
@@ -5976,7 +5976,7 @@
       <c r="G226" s="2"/>
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="1:8">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A227" s="2"/>
       <c r="B227" s="2"/>
       <c r="C227" s="2"/>
@@ -5988,7 +5988,7 @@
       <c r="G227" s="2"/>
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="1:8">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A228" s="2" t="s">
         <v>131</v>
       </c>
@@ -6004,7 +6004,7 @@
       <c r="G228" s="2"/>
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="1:8">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A229" s="2"/>
       <c r="B229" s="2"/>
       <c r="C229" s="2"/>
@@ -6016,7 +6016,7 @@
       <c r="G229" s="2"/>
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="1:8">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A230" s="2"/>
       <c r="B230" s="2"/>
       <c r="C230" s="2"/>
@@ -6028,7 +6028,7 @@
       <c r="G230" s="2"/>
       <c r="H230" s="2"/>
     </row>
-    <row r="231" spans="1:8">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A231" s="2"/>
       <c r="B231" s="2"/>
       <c r="C231" s="2"/>
@@ -6040,7 +6040,7 @@
       <c r="G231" s="2"/>
       <c r="H231" s="2"/>
     </row>
-    <row r="232" spans="1:8">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
         <v>180</v>
       </c>
@@ -6052,7 +6052,7 @@
       <c r="G232" s="1"/>
       <c r="H232" s="1"/>
     </row>
-    <row r="233" spans="1:8">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A233" s="1"/>
       <c r="B233" s="1" t="s">
         <v>181</v>
@@ -6066,7 +6066,7 @@
       <c r="G233" s="1"/>
       <c r="H233" s="1"/>
     </row>
-    <row r="234" spans="1:8">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A234" s="1"/>
       <c r="B234" s="1"/>
       <c r="C234" s="1"/>
@@ -6078,7 +6078,7 @@
       <c r="G234" s="1"/>
       <c r="H234" s="1"/>
     </row>
-    <row r="235" spans="1:8">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
         <v>131</v>
       </c>
@@ -6094,7 +6094,7 @@
       <c r="G235" s="1"/>
       <c r="H235" s="1"/>
     </row>
-    <row r="236" spans="1:8">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A236" s="1"/>
       <c r="B236" s="1"/>
       <c r="C236" s="1"/>
@@ -6106,7 +6106,7 @@
       <c r="G236" s="1"/>
       <c r="H236" s="1"/>
     </row>
-    <row r="237" spans="1:8">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A237" s="1"/>
       <c r="B237" s="1"/>
       <c r="C237" s="1"/>
@@ -6118,7 +6118,7 @@
       <c r="G237" s="1"/>
       <c r="H237" s="1"/>
     </row>
-    <row r="238" spans="1:8">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A238" s="1"/>
       <c r="B238" s="1" t="s">
         <v>183</v>
@@ -6132,7 +6132,7 @@
       <c r="G238" s="1"/>
       <c r="H238" s="1"/>
     </row>
-    <row r="239" spans="1:8">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A239" s="1"/>
       <c r="B239" s="1"/>
       <c r="C239" s="1"/>
@@ -6144,7 +6144,7 @@
       <c r="G239" s="1"/>
       <c r="H239" s="1"/>
     </row>
-    <row r="240" spans="1:8">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A240" s="1"/>
       <c r="B240" s="1"/>
       <c r="C240" s="1"/>
@@ -6156,7 +6156,7 @@
       <c r="G240" s="1"/>
       <c r="H240" s="1"/>
     </row>
-    <row r="241" spans="1:8">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A241" s="2" t="s">
         <v>36</v>
       </c>
@@ -6170,7 +6170,7 @@
       <c r="G241" s="2"/>
       <c r="H241" s="2"/>
     </row>
-    <row r="242" spans="1:8">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A242" s="2" t="s">
         <v>131</v>
       </c>
@@ -6184,7 +6184,7 @@
       <c r="G242" s="2"/>
       <c r="H242" s="2"/>
     </row>
-    <row r="243" spans="1:8">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
         <v>184</v>
       </c>
@@ -6198,7 +6198,7 @@
       <c r="G243" s="1"/>
       <c r="H243" s="1"/>
     </row>
-    <row r="244" spans="1:8">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="s">
         <v>131</v>
       </c>
@@ -6214,7 +6214,7 @@
       <c r="G244" s="1"/>
       <c r="H244" s="1"/>
     </row>
-    <row r="245" spans="1:8">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A245" s="1"/>
       <c r="B245" s="1"/>
       <c r="C245" s="1"/>
@@ -6436,28 +6436,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AMJ195"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="2" max="2" width="12.5" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" style="22" customWidth="1"/>
-    <col min="6" max="6" width="43.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" customWidth="1"/>
-    <col min="9" max="9" width="6.85546875" customWidth="1"/>
-    <col min="10" max="10" width="36.140625" customWidth="1"/>
-    <col min="11" max="11" width="37.7109375" customWidth="1"/>
-    <col min="12" max="12" width="45.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="5" max="5" width="18.5" style="22" customWidth="1"/>
+    <col min="6" max="6" width="43.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.5" customWidth="1"/>
+    <col min="9" max="9" width="6.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.1640625" customWidth="1"/>
+    <col min="11" max="11" width="37.6640625" customWidth="1"/>
+    <col min="12" max="12" width="45.1640625" customWidth="1"/>
     <col min="13" max="13" width="41" customWidth="1"/>
-    <col min="14" max="14" width="32.7109375" customWidth="1"/>
+    <col min="14" max="14" width="32.6640625" customWidth="1"/>
     <col min="15" max="15" width="32" customWidth="1"/>
-    <col min="16" max="16" width="63.7109375" customWidth="1"/>
-    <col min="1024" max="1024" width="11.42578125" customWidth="1"/>
+    <col min="16" max="16" width="63.6640625" customWidth="1"/>
+    <col min="1024" max="1024" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="30">
+    <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>186</v>
       </c>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="Q1" s="24"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="25">
         <v>2</v>
       </c>
@@ -6536,7 +6536,7 @@
       <c r="O2" s="5"/>
       <c r="R2" s="13"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="28">
         <v>4</v>
       </c>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="Q3" s="35"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="28">
         <v>5</v>
       </c>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="Q4" s="35"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="28"/>
       <c r="B5" s="21"/>
       <c r="C5" s="28">
@@ -6645,7 +6645,7 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="35"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="36">
         <v>6</v>
       </c>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="Q6" s="35"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="36"/>
       <c r="B7" s="3"/>
       <c r="C7" s="36">
@@ -6715,7 +6715,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="35"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="36"/>
       <c r="B8" s="3"/>
       <c r="C8" s="36">
@@ -6742,7 +6742,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="35"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="36">
         <v>7</v>
       </c>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="Q9" s="42"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="36"/>
       <c r="B10" s="3"/>
       <c r="C10" s="36">
@@ -6812,7 +6812,7 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="42"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="36"/>
       <c r="B11" s="3"/>
       <c r="C11" s="36">
@@ -6839,7 +6839,7 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="42"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="28">
         <v>210</v>
       </c>
@@ -6872,7 +6872,7 @@
       </c>
       <c r="Q12" s="35"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="28">
         <v>8</v>
       </c>
@@ -6909,7 +6909,7 @@
       </c>
       <c r="Q13" s="35"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="28">
         <v>9</v>
       </c>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="Q14" s="42"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="28"/>
       <c r="B15" s="21"/>
       <c r="C15" s="28">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="Q15" s="42"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="28"/>
       <c r="B16" s="21"/>
       <c r="C16" s="28">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="Q16" s="42"/>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="28">
         <v>10</v>
       </c>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="Q17" s="35"/>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="28">
         <v>11</v>
       </c>
@@ -7090,7 +7090,7 @@
       </c>
       <c r="Q18" s="35"/>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="28">
         <v>12</v>
       </c>
@@ -7133,7 +7133,7 @@
       </c>
       <c r="Q19" s="35"/>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="28"/>
       <c r="B20" s="21"/>
       <c r="C20" s="28">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="Q20" s="35"/>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="28">
         <v>13</v>
       </c>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="Q21" s="35"/>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="28">
         <v>14</v>
       </c>
@@ -7248,7 +7248,7 @@
       </c>
       <c r="Q22" s="35"/>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="28"/>
       <c r="B23" s="21"/>
       <c r="C23" s="28">
@@ -7275,7 +7275,7 @@
       <c r="P23" s="2"/>
       <c r="Q23" s="35"/>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="28">
         <v>16</v>
       </c>
@@ -7318,7 +7318,7 @@
       </c>
       <c r="Q24" s="35"/>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="28">
         <v>17</v>
       </c>
@@ -7361,7 +7361,7 @@
       </c>
       <c r="Q25" s="35"/>
     </row>
-    <row r="26" spans="1:17">
+    <row r="26" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="28"/>
       <c r="B26" s="21"/>
       <c r="C26" s="28">
@@ -7388,7 +7388,7 @@
       <c r="P26" s="2"/>
       <c r="Q26" s="35"/>
     </row>
-    <row r="27" spans="1:17">
+    <row r="27" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="28">
         <v>15</v>
       </c>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="D27" s="21"/>
       <c r="E27" s="88" t="s">
-        <v>615</v>
+        <v>659</v>
       </c>
       <c r="F27" s="46" t="s">
         <v>100</v>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="Q27" s="35"/>
     </row>
-    <row r="28" spans="1:17">
+    <row r="28" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="28"/>
       <c r="B28" s="21"/>
       <c r="C28" s="28">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="D28" s="21"/>
       <c r="E28" s="88" t="s">
-        <v>615</v>
+        <v>659</v>
       </c>
       <c r="F28" s="46" t="s">
         <v>100</v>
@@ -7458,7 +7458,7 @@
       <c r="P28" s="2"/>
       <c r="Q28" s="35"/>
     </row>
-    <row r="29" spans="1:17">
+    <row r="29" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="28"/>
       <c r="B29" s="21"/>
       <c r="C29" s="28">
@@ -7466,7 +7466,7 @@
       </c>
       <c r="D29" s="21"/>
       <c r="E29" s="88" t="s">
-        <v>615</v>
+        <v>659</v>
       </c>
       <c r="F29" s="46" t="s">
         <v>100</v>
@@ -7485,7 +7485,7 @@
       <c r="P29" s="2"/>
       <c r="Q29" s="35"/>
     </row>
-    <row r="30" spans="1:17" s="72" customFormat="1">
+    <row r="30" spans="1:17" s="72" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="66">
         <v>201</v>
       </c>
@@ -7516,7 +7516,7 @@
       </c>
       <c r="Q30" s="71"/>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="36">
         <v>18</v>
       </c>
@@ -7526,7 +7526,7 @@
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="89" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>102</v>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="Q31" s="35"/>
     </row>
-    <row r="32" spans="1:17">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" s="36">
         <v>19</v>
       </c>
@@ -7567,7 +7567,7 @@
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="89" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="F32" s="41" t="s">
         <v>103</v>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="Q32" s="42"/>
     </row>
-    <row r="33" spans="1:1024">
+    <row r="33" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A33" s="36"/>
       <c r="B33" s="3"/>
       <c r="C33" s="36">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="89" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="F33" s="41" t="s">
         <v>103</v>
@@ -7629,7 +7629,7 @@
       </c>
       <c r="Q33" s="42"/>
     </row>
-    <row r="34" spans="1:1024">
+    <row r="34" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A34" s="36"/>
       <c r="B34" s="3"/>
       <c r="C34" s="36">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="89" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="F34" s="41" t="s">
         <v>103</v>
@@ -7660,7 +7660,7 @@
       </c>
       <c r="Q34" s="42"/>
     </row>
-    <row r="35" spans="1:1024">
+    <row r="35" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="36">
         <v>20</v>
       </c>
@@ -7670,7 +7670,7 @@
       <c r="C35" s="36"/>
       <c r="D35" s="3"/>
       <c r="E35" s="89" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="F35" s="41" t="s">
         <v>105</v>
@@ -7695,7 +7695,7 @@
       </c>
       <c r="Q35" s="35"/>
     </row>
-    <row r="36" spans="1:1024">
+    <row r="36" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="36">
         <v>21</v>
       </c>
@@ -7705,7 +7705,7 @@
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="89" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F36" s="49" t="s">
         <v>251</v>
@@ -7736,7 +7736,7 @@
       </c>
       <c r="Q36" s="35"/>
     </row>
-    <row r="37" spans="1:1024">
+    <row r="37" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="36"/>
       <c r="B37" s="3"/>
       <c r="C37" s="36">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="89" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F37" s="49" t="s">
         <v>251</v>
@@ -7767,7 +7767,7 @@
       </c>
       <c r="Q37" s="35"/>
     </row>
-    <row r="38" spans="1:1024">
+    <row r="38" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A38" s="36">
         <v>22</v>
       </c>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="89" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="F38" s="49" t="s">
         <v>256</v>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="Q38" s="42"/>
     </row>
-    <row r="39" spans="1:1024">
+    <row r="39" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A39" s="36"/>
       <c r="B39" s="3"/>
       <c r="C39" s="36">
@@ -7818,7 +7818,7 @@
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="89" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="F39" s="49" t="s">
         <v>256</v>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="Q39" s="42"/>
     </row>
-    <row r="40" spans="1:1024">
+    <row r="40" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A40" s="36"/>
       <c r="B40" s="3"/>
       <c r="C40" s="36">
@@ -7849,7 +7849,7 @@
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="89" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="F40" s="49" t="s">
         <v>256</v>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="Q40" s="42"/>
     </row>
-    <row r="41" spans="1:1024" s="85" customFormat="1">
+    <row r="41" spans="1:1024" s="85" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="50">
         <v>211</v>
       </c>
@@ -7906,7 +7906,7 @@
       <c r="Q41" s="84"/>
       <c r="AMJ41" s="86"/>
     </row>
-    <row r="42" spans="1:1024" s="85" customFormat="1">
+    <row r="42" spans="1:1024" s="85" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="50">
         <v>39</v>
       </c>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="D42" s="51"/>
       <c r="E42" s="90" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="F42" s="51" t="s">
         <v>126</v>
@@ -7942,7 +7942,7 @@
       <c r="Q42" s="84"/>
       <c r="AMJ42" s="86"/>
     </row>
-    <row r="43" spans="1:1024" s="55" customFormat="1">
+    <row r="43" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="50">
         <v>40</v>
       </c>
@@ -7954,7 +7954,7 @@
       </c>
       <c r="D43" s="51"/>
       <c r="E43" s="90" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="F43" s="56" t="s">
         <v>127</v>
@@ -7986,7 +7986,7 @@
       <c r="Q43" s="57"/>
       <c r="AMJ43"/>
     </row>
-    <row r="44" spans="1:1024" s="55" customFormat="1">
+    <row r="44" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="50"/>
       <c r="B44" s="51"/>
       <c r="C44" s="50">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="D44" s="51"/>
       <c r="E44" s="90" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="F44" s="56" t="s">
         <v>127</v>
@@ -8018,7 +8018,7 @@
       <c r="Q44" s="57"/>
       <c r="AMJ44"/>
     </row>
-    <row r="45" spans="1:1024" s="55" customFormat="1">
+    <row r="45" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="50"/>
       <c r="B45" s="51"/>
       <c r="C45" s="50">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="D45" s="51"/>
       <c r="E45" s="90" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="F45" s="56" t="s">
         <v>127</v>
@@ -8050,7 +8050,7 @@
       <c r="Q45" s="57"/>
       <c r="AMJ45"/>
     </row>
-    <row r="46" spans="1:1024" s="55" customFormat="1">
+    <row r="46" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="50">
         <v>41</v>
       </c>
@@ -8062,7 +8062,7 @@
       </c>
       <c r="D46" s="51"/>
       <c r="E46" s="90" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F46" s="56" t="s">
         <v>128</v>
@@ -8092,7 +8092,7 @@
       <c r="Q46" s="57"/>
       <c r="AMJ46"/>
     </row>
-    <row r="47" spans="1:1024" s="55" customFormat="1">
+    <row r="47" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="50"/>
       <c r="B47" s="51"/>
       <c r="C47" s="50">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="D47" s="51"/>
       <c r="E47" s="90" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F47" s="56" t="s">
         <v>128</v>
@@ -8124,7 +8124,7 @@
       <c r="Q47" s="57"/>
       <c r="AMJ47"/>
     </row>
-    <row r="48" spans="1:1024" s="55" customFormat="1">
+    <row r="48" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="50">
         <v>42</v>
       </c>
@@ -8136,7 +8136,7 @@
       </c>
       <c r="D48" s="51"/>
       <c r="E48" s="90" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="F48" s="56" t="s">
         <v>129</v>
@@ -8166,7 +8166,7 @@
       <c r="Q48" s="57"/>
       <c r="AMJ48"/>
     </row>
-    <row r="49" spans="1:1024" s="80" customFormat="1">
+    <row r="49" spans="1:1024" s="80" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="73">
         <v>202</v>
       </c>
@@ -8196,7 +8196,7 @@
       <c r="Q49" s="79"/>
       <c r="AMJ49" s="81"/>
     </row>
-    <row r="50" spans="1:1024" s="55" customFormat="1">
+    <row r="50" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="28">
         <v>23</v>
       </c>
@@ -8206,7 +8206,7 @@
       </c>
       <c r="D50" s="21"/>
       <c r="E50" s="88" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="F50" s="21" t="s">
         <v>108</v>
@@ -8236,7 +8236,7 @@
       <c r="Q50" s="54"/>
       <c r="AMJ50"/>
     </row>
-    <row r="51" spans="1:1024" s="55" customFormat="1">
+    <row r="51" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="28"/>
       <c r="B51" s="21"/>
       <c r="C51" s="28">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="D51" s="21"/>
       <c r="E51" s="88" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="F51" s="21" t="s">
         <v>108</v>
@@ -8268,7 +8268,7 @@
       <c r="Q51" s="54"/>
       <c r="AMJ51"/>
     </row>
-    <row r="52" spans="1:1024" s="55" customFormat="1">
+    <row r="52" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="28"/>
       <c r="B52" s="21"/>
       <c r="C52" s="28">
@@ -8276,7 +8276,7 @@
       </c>
       <c r="D52" s="21"/>
       <c r="E52" s="88" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="F52" s="21" t="s">
         <v>108</v>
@@ -8304,7 +8304,7 @@
       <c r="Q52" s="54"/>
       <c r="AMJ52"/>
     </row>
-    <row r="53" spans="1:1024" s="55" customFormat="1">
+    <row r="53" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="28"/>
       <c r="B53" s="21"/>
       <c r="C53" s="28">
@@ -8342,7 +8342,7 @@
       <c r="Q53" s="54"/>
       <c r="AMJ53"/>
     </row>
-    <row r="54" spans="1:1024" s="55" customFormat="1">
+    <row r="54" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="28">
         <v>24</v>
       </c>
@@ -8354,7 +8354,7 @@
       </c>
       <c r="D54" s="21"/>
       <c r="E54" s="88" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="F54" s="33" t="s">
         <v>595</v>
@@ -8386,7 +8386,7 @@
       <c r="Q54" s="54"/>
       <c r="AMJ54"/>
     </row>
-    <row r="55" spans="1:1024" s="55" customFormat="1">
+    <row r="55" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="28">
         <v>25</v>
       </c>
@@ -8398,7 +8398,7 @@
       </c>
       <c r="D55" s="21"/>
       <c r="E55" s="88" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F55" s="33" t="s">
         <v>111</v>
@@ -8430,7 +8430,7 @@
       <c r="Q55" s="54"/>
       <c r="AMJ55"/>
     </row>
-    <row r="56" spans="1:1024" s="55" customFormat="1">
+    <row r="56" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="28"/>
       <c r="B56" s="21"/>
       <c r="C56" s="28">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="D56" s="21"/>
       <c r="E56" s="88" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F56" s="33" t="s">
         <v>111</v>
@@ -8462,7 +8462,7 @@
       <c r="Q56" s="54"/>
       <c r="AMJ56"/>
     </row>
-    <row r="57" spans="1:1024" s="55" customFormat="1">
+    <row r="57" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="28"/>
       <c r="B57" s="21"/>
       <c r="C57" s="28">
@@ -8470,7 +8470,7 @@
       </c>
       <c r="D57" s="21"/>
       <c r="E57" s="88" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F57" s="33" t="s">
         <v>111</v>
@@ -8494,7 +8494,7 @@
       <c r="Q57" s="54"/>
       <c r="AMJ57"/>
     </row>
-    <row r="58" spans="1:1024" s="55" customFormat="1">
+    <row r="58" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="28">
         <v>26</v>
       </c>
@@ -8506,7 +8506,7 @@
       </c>
       <c r="D58" s="21"/>
       <c r="E58" s="88" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F58" s="58" t="s">
         <v>112</v>
@@ -8539,7 +8539,7 @@
       </c>
       <c r="AMJ58"/>
     </row>
-    <row r="59" spans="1:1024" s="55" customFormat="1">
+    <row r="59" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="28"/>
       <c r="B59" s="21"/>
       <c r="C59" s="28">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="D59" s="21"/>
       <c r="E59" s="88" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F59" s="58" t="s">
         <v>112</v>
@@ -8570,7 +8570,7 @@
       </c>
       <c r="AMJ59"/>
     </row>
-    <row r="60" spans="1:1024" s="55" customFormat="1">
+    <row r="60" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="28"/>
       <c r="B60" s="21"/>
       <c r="C60" s="28">
@@ -8578,7 +8578,7 @@
       </c>
       <c r="D60" s="21"/>
       <c r="E60" s="88" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F60" s="33" t="s">
         <v>113</v>
@@ -8604,7 +8604,7 @@
       <c r="Q60" s="54"/>
       <c r="AMJ60"/>
     </row>
-    <row r="61" spans="1:1024" s="55" customFormat="1">
+    <row r="61" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="28">
         <v>27</v>
       </c>
@@ -8616,7 +8616,7 @@
       </c>
       <c r="D61" s="21"/>
       <c r="E61" s="88" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F61" s="33" t="s">
         <v>114</v>
@@ -8648,7 +8648,7 @@
       <c r="Q61" s="54"/>
       <c r="AMJ61"/>
     </row>
-    <row r="62" spans="1:1024" s="55" customFormat="1">
+    <row r="62" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="28">
         <v>28</v>
       </c>
@@ -8660,7 +8660,7 @@
       </c>
       <c r="D62" s="21"/>
       <c r="E62" s="88" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="F62" s="33" t="s">
         <v>73</v>
@@ -8692,7 +8692,7 @@
       <c r="Q62" s="54"/>
       <c r="AMJ62"/>
     </row>
-    <row r="63" spans="1:1024" s="55" customFormat="1">
+    <row r="63" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="28"/>
       <c r="B63" s="21"/>
       <c r="C63" s="28">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="D63" s="21"/>
       <c r="E63" s="88" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="F63" s="33" t="s">
         <v>73</v>
@@ -8724,7 +8724,7 @@
       <c r="Q63" s="54"/>
       <c r="AMJ63"/>
     </row>
-    <row r="64" spans="1:1024" s="55" customFormat="1">
+    <row r="64" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="28"/>
       <c r="B64" s="21"/>
       <c r="C64" s="28">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="D64" s="21"/>
       <c r="E64" s="88" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="F64" s="33" t="s">
         <v>73</v>
@@ -8756,7 +8756,7 @@
       <c r="Q64" s="54"/>
       <c r="AMJ64"/>
     </row>
-    <row r="65" spans="1:1024" s="55" customFormat="1" ht="30">
+    <row r="65" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="36">
         <v>212</v>
       </c>
@@ -8790,7 +8790,7 @@
       <c r="Q65" s="54"/>
       <c r="AMJ65"/>
     </row>
-    <row r="66" spans="1:1024" s="55" customFormat="1" ht="30">
+    <row r="66" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="36">
         <v>29</v>
       </c>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="D66" s="3"/>
       <c r="E66" s="89" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F66" s="37" t="s">
         <v>115</v>
@@ -8832,7 +8832,7 @@
       <c r="Q66" s="54"/>
       <c r="AMJ66"/>
     </row>
-    <row r="67" spans="1:1024" s="55" customFormat="1">
+    <row r="67" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="36">
         <v>30</v>
       </c>
@@ -8842,7 +8842,7 @@
       </c>
       <c r="D67" s="3"/>
       <c r="E67" s="89" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F67" s="59" t="s">
         <v>117</v>
@@ -8874,7 +8874,7 @@
       <c r="Q67" s="57"/>
       <c r="AMJ67"/>
     </row>
-    <row r="68" spans="1:1024" s="55" customFormat="1">
+    <row r="68" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="36"/>
       <c r="B68" s="3"/>
       <c r="C68" s="36">
@@ -8882,7 +8882,7 @@
       </c>
       <c r="D68" s="3"/>
       <c r="E68" s="89" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F68" s="59" t="s">
         <v>117</v>
@@ -8906,7 +8906,7 @@
       <c r="Q68" s="57"/>
       <c r="AMJ68"/>
     </row>
-    <row r="69" spans="1:1024" s="55" customFormat="1">
+    <row r="69" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="50">
         <v>34</v>
       </c>
@@ -8954,7 +8954,7 @@
       <c r="Q69" s="54"/>
       <c r="AMJ69"/>
     </row>
-    <row r="70" spans="1:1024" s="55" customFormat="1">
+    <row r="70" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="50"/>
       <c r="B70" s="51"/>
       <c r="C70" s="50">
@@ -8986,7 +8986,7 @@
       <c r="Q70" s="54"/>
       <c r="AMJ70"/>
     </row>
-    <row r="71" spans="1:1024" s="55" customFormat="1">
+    <row r="71" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="50"/>
       <c r="B71" s="51"/>
       <c r="C71" s="50">
@@ -9018,7 +9018,7 @@
       <c r="Q71" s="54"/>
       <c r="AMJ71"/>
     </row>
-    <row r="72" spans="1:1024" s="55" customFormat="1">
+    <row r="72" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="50"/>
       <c r="B72" s="51"/>
       <c r="C72" s="50">
@@ -9052,7 +9052,7 @@
       <c r="Q72" s="54"/>
       <c r="AMJ72"/>
     </row>
-    <row r="73" spans="1:1024" s="55" customFormat="1">
+    <row r="73" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="50"/>
       <c r="B73" s="51"/>
       <c r="C73" s="50">
@@ -9090,12 +9090,12 @@
       <c r="Q73" s="57"/>
       <c r="AMJ73"/>
     </row>
-    <row r="74" spans="1:1024" s="55" customFormat="1">
+    <row r="74" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A74" s="28">
         <v>31</v>
       </c>
       <c r="B74" s="88" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C74" s="28"/>
       <c r="D74" s="21"/>
@@ -9122,7 +9122,7 @@
       <c r="Q74" s="54"/>
       <c r="AMJ74"/>
     </row>
-    <row r="75" spans="1:1024" s="55" customFormat="1">
+    <row r="75" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A75" s="28">
         <v>32</v>
       </c>
@@ -9164,7 +9164,7 @@
       <c r="Q75" s="54"/>
       <c r="AMJ75"/>
     </row>
-    <row r="76" spans="1:1024" s="55" customFormat="1">
+    <row r="76" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="28"/>
       <c r="B76" s="21"/>
       <c r="C76" s="28">
@@ -9196,7 +9196,7 @@
       <c r="Q76" s="54"/>
       <c r="AMJ76"/>
     </row>
-    <row r="77" spans="1:1024" s="55" customFormat="1">
+    <row r="77" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="28"/>
       <c r="B77" s="21"/>
       <c r="C77" s="28">
@@ -9234,7 +9234,7 @@
       <c r="Q77" s="57"/>
       <c r="AMJ77"/>
     </row>
-    <row r="78" spans="1:1024" s="55" customFormat="1">
+    <row r="78" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="28">
         <v>33</v>
       </c>
@@ -9276,7 +9276,7 @@
       <c r="Q78" s="54"/>
       <c r="AMJ78"/>
     </row>
-    <row r="79" spans="1:1024" s="55" customFormat="1">
+    <row r="79" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="36">
         <v>35</v>
       </c>
@@ -9310,7 +9310,7 @@
       <c r="Q79" s="54"/>
       <c r="AMJ79"/>
     </row>
-    <row r="80" spans="1:1024" s="55" customFormat="1">
+    <row r="80" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="36">
         <v>36</v>
       </c>
@@ -9354,7 +9354,7 @@
       <c r="Q80" s="57"/>
       <c r="AMJ80"/>
     </row>
-    <row r="81" spans="1:1024" s="55" customFormat="1">
+    <row r="81" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="36"/>
       <c r="B81" s="3"/>
       <c r="C81" s="36">
@@ -9386,7 +9386,7 @@
       <c r="Q81" s="57"/>
       <c r="AMJ81"/>
     </row>
-    <row r="82" spans="1:1024" s="55" customFormat="1">
+    <row r="82" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="36"/>
       <c r="B82" s="3"/>
       <c r="C82" s="36">
@@ -9418,7 +9418,7 @@
       <c r="Q82" s="57"/>
       <c r="AMJ82"/>
     </row>
-    <row r="83" spans="1:1024" s="55" customFormat="1">
+    <row r="83" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="36">
         <v>37</v>
       </c>
@@ -9458,7 +9458,7 @@
       <c r="Q83" s="57"/>
       <c r="AMJ83"/>
     </row>
-    <row r="84" spans="1:1024" s="55" customFormat="1">
+    <row r="84" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="36"/>
       <c r="B84" s="3"/>
       <c r="C84" s="36">
@@ -9490,7 +9490,7 @@
       <c r="Q84" s="57"/>
       <c r="AMJ84"/>
     </row>
-    <row r="85" spans="1:1024" s="55" customFormat="1">
+    <row r="85" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="36"/>
       <c r="B85" s="3"/>
       <c r="C85" s="36">
@@ -9522,7 +9522,7 @@
       <c r="Q85" s="57"/>
       <c r="AMJ85"/>
     </row>
-    <row r="86" spans="1:1024" s="55" customFormat="1">
+    <row r="86" spans="1:1024" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="36"/>
       <c r="B86" s="3"/>
       <c r="C86" s="36">
@@ -9554,7 +9554,7 @@
       <c r="Q86" s="54"/>
       <c r="AMJ86"/>
     </row>
-    <row r="87" spans="1:1024" s="55" customFormat="1">
+    <row r="87" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="36">
         <v>38</v>
       </c>
@@ -9598,7 +9598,7 @@
       <c r="Q87" s="57"/>
       <c r="AMJ87"/>
     </row>
-    <row r="88" spans="1:1024" s="55" customFormat="1">
+    <row r="88" spans="1:1024" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A88" s="36"/>
       <c r="B88" s="3"/>
       <c r="C88" s="36">
@@ -9630,7 +9630,7 @@
       <c r="Q88" s="57"/>
       <c r="AMJ88"/>
     </row>
-    <row r="89" spans="1:1024">
+    <row r="89" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A89" s="61">
         <v>43</v>
       </c>
@@ -9657,7 +9657,7 @@
       <c r="N89" s="63"/>
       <c r="Q89" s="42"/>
     </row>
-    <row r="90" spans="1:1024">
+    <row r="90" spans="1:1024" ht="16" x14ac:dyDescent="0.2">
       <c r="A90" s="28">
         <v>44</v>
       </c>
@@ -9696,7 +9696,7 @@
       </c>
       <c r="Q90" s="42"/>
     </row>
-    <row r="91" spans="1:1024">
+    <row r="91" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A91" s="36">
         <v>45</v>
       </c>
@@ -9733,7 +9733,7 @@
       </c>
       <c r="Q91" s="42"/>
     </row>
-    <row r="92" spans="1:1024">
+    <row r="92" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A92" s="28">
         <v>204</v>
       </c>
@@ -9764,7 +9764,7 @@
       </c>
       <c r="Q92" s="42"/>
     </row>
-    <row r="93" spans="1:1024">
+    <row r="93" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A93" s="28">
         <v>46</v>
       </c>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D93" s="21"/>
       <c r="E93" s="88" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F93" s="21" t="s">
         <v>92</v>
@@ -9801,7 +9801,7 @@
       </c>
       <c r="Q93" s="42"/>
     </row>
-    <row r="94" spans="1:1024">
+    <row r="94" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A94" s="28">
         <v>47</v>
       </c>
@@ -9813,7 +9813,7 @@
       </c>
       <c r="D94" s="21"/>
       <c r="E94" s="88" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F94" s="33" t="s">
         <v>133</v>
@@ -9840,7 +9840,7 @@
       </c>
       <c r="Q94" s="42"/>
     </row>
-    <row r="95" spans="1:1024">
+    <row r="95" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A95" s="28">
         <v>48</v>
       </c>
@@ -9852,7 +9852,7 @@
       </c>
       <c r="D95" s="21"/>
       <c r="E95" s="88" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="F95" s="33" t="s">
         <v>134</v>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="Q95" s="42"/>
     </row>
-    <row r="96" spans="1:1024">
+    <row r="96" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A96" s="28">
         <v>49</v>
       </c>
@@ -9891,7 +9891,7 @@
       </c>
       <c r="D96" s="21"/>
       <c r="E96" s="88" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F96" s="33" t="s">
         <v>135</v>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="Q96" s="42"/>
     </row>
-    <row r="97" spans="1:17">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A97" s="28">
         <v>50</v>
       </c>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D97" s="21"/>
       <c r="E97" s="88" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F97" s="33" t="s">
         <v>97</v>
@@ -9957,7 +9957,7 @@
       </c>
       <c r="Q97" s="42"/>
     </row>
-    <row r="98" spans="1:17">
+    <row r="98" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A98" s="28">
         <v>54</v>
       </c>
@@ -9969,7 +9969,7 @@
       </c>
       <c r="D98" s="21"/>
       <c r="E98" s="88" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="F98" s="33" t="s">
         <v>138</v>
@@ -9998,7 +9998,7 @@
       </c>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" spans="1:17">
+    <row r="99" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A99" s="28">
         <v>55</v>
       </c>
@@ -10010,7 +10010,7 @@
       </c>
       <c r="D99" s="21"/>
       <c r="E99" s="88" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="F99" s="33" t="s">
         <v>139</v>
@@ -10039,7 +10039,7 @@
       </c>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" spans="1:17">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A100" s="36">
         <v>56</v>
       </c>
@@ -10080,7 +10080,7 @@
       </c>
       <c r="Q100" s="42"/>
     </row>
-    <row r="101" spans="1:17">
+    <row r="101" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="28">
         <v>57</v>
       </c>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" spans="1:17">
+    <row r="102" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A102" s="28">
         <v>58</v>
       </c>
@@ -10150,7 +10150,7 @@
       </c>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" spans="1:17">
+    <row r="103" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A103" s="28">
         <v>59</v>
       </c>
@@ -10191,7 +10191,7 @@
       </c>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" spans="1:17">
+    <row r="104" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A104" s="28">
         <v>60</v>
       </c>
@@ -10232,7 +10232,7 @@
       </c>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" spans="1:17">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A105" s="28">
         <v>61</v>
       </c>
@@ -10273,7 +10273,7 @@
       </c>
       <c r="Q105" s="42"/>
     </row>
-    <row r="106" spans="1:17">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A106" s="28">
         <v>205</v>
       </c>
@@ -10285,7 +10285,7 @@
       </c>
       <c r="D106" s="21"/>
       <c r="E106" s="88" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F106" s="33" t="s">
         <v>145</v>
@@ -10312,7 +10312,7 @@
       </c>
       <c r="Q106" s="42"/>
     </row>
-    <row r="107" spans="1:17">
+    <row r="107" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" s="36">
         <v>62</v>
       </c>
@@ -10343,7 +10343,7 @@
       </c>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" spans="1:17">
+    <row r="108" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A108" s="36">
         <v>63</v>
       </c>
@@ -10382,7 +10382,7 @@
       </c>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" spans="1:17">
+    <row r="109" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A109" s="36"/>
       <c r="B109" s="3"/>
       <c r="C109" s="36">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" spans="1:17">
+    <row r="110" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A110" s="36"/>
       <c r="B110" s="3"/>
       <c r="C110" s="36">
@@ -10440,7 +10440,7 @@
       </c>
       <c r="Q110" s="35"/>
     </row>
-    <row r="111" spans="1:17">
+    <row r="111" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A111" s="36">
         <v>64</v>
       </c>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="Q111" s="35"/>
     </row>
-    <row r="112" spans="1:17">
+    <row r="112" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A112" s="36"/>
       <c r="B112" s="3"/>
       <c r="C112" s="36">
@@ -10510,7 +10510,7 @@
       </c>
       <c r="Q112" s="35"/>
     </row>
-    <row r="113" spans="1:17">
+    <row r="113" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A113" s="36">
         <v>65</v>
       </c>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="Q113" s="35"/>
     </row>
-    <row r="114" spans="1:17">
+    <row r="114" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A114" s="36"/>
       <c r="B114" s="3"/>
       <c r="C114" s="36">
@@ -10584,7 +10584,7 @@
       </c>
       <c r="Q114" s="35"/>
     </row>
-    <row r="115" spans="1:17">
+    <row r="115" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A115" s="36">
         <v>66</v>
       </c>
@@ -10623,7 +10623,7 @@
       </c>
       <c r="Q115" s="35"/>
     </row>
-    <row r="116" spans="1:17">
+    <row r="116" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A116" s="36">
         <v>67</v>
       </c>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="Q116" s="35"/>
     </row>
-    <row r="117" spans="1:17">
+    <row r="117" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A117" s="36"/>
       <c r="B117" s="3"/>
       <c r="C117" s="36">
@@ -10691,7 +10691,7 @@
       <c r="P117" s="1"/>
       <c r="Q117" s="35"/>
     </row>
-    <row r="118" spans="1:17">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A118" s="36"/>
       <c r="B118" s="3"/>
       <c r="C118" s="36">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="Q118" s="42"/>
     </row>
-    <row r="119" spans="1:17">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A119" s="28">
         <v>68</v>
       </c>
@@ -10757,7 +10757,7 @@
       </c>
       <c r="Q119" s="42"/>
     </row>
-    <row r="120" spans="1:17">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A120" s="28">
         <v>203</v>
       </c>
@@ -10786,7 +10786,7 @@
       </c>
       <c r="Q120" s="42"/>
     </row>
-    <row r="121" spans="1:17">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A121" s="28">
         <v>51</v>
       </c>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="D121" s="21"/>
       <c r="E121" s="88" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F121" s="33" t="s">
         <v>93</v>
@@ -10825,7 +10825,7 @@
       </c>
       <c r="Q121" s="42"/>
     </row>
-    <row r="122" spans="1:17">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A122" s="28">
         <v>52</v>
       </c>
@@ -10837,7 +10837,7 @@
       </c>
       <c r="D122" s="21"/>
       <c r="E122" s="88" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="F122" s="46" t="s">
         <v>377</v>
@@ -10864,7 +10864,7 @@
       </c>
       <c r="Q122" s="42"/>
     </row>
-    <row r="123" spans="1:17">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A123" s="28"/>
       <c r="B123" s="21"/>
       <c r="C123" s="28">
@@ -10872,7 +10872,7 @@
       </c>
       <c r="D123" s="21"/>
       <c r="E123" s="88" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="F123" s="46" t="s">
         <v>377</v>
@@ -10893,7 +10893,7 @@
       </c>
       <c r="Q123" s="42"/>
     </row>
-    <row r="124" spans="1:17">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A124" s="28"/>
       <c r="B124" s="21"/>
       <c r="C124" s="28">
@@ -10901,7 +10901,7 @@
       </c>
       <c r="D124" s="21"/>
       <c r="E124" s="88" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="F124" s="46" t="s">
         <v>377</v>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="Q124" s="42"/>
     </row>
-    <row r="125" spans="1:17">
+    <row r="125" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A125" s="28">
         <v>53</v>
       </c>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="D125" s="21"/>
       <c r="E125" s="88" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F125" s="46" t="s">
         <v>160</v>
@@ -10961,7 +10961,7 @@
       </c>
       <c r="Q125" s="35"/>
     </row>
-    <row r="126" spans="1:17">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A126" s="28">
         <v>213</v>
       </c>
@@ -10990,7 +10990,7 @@
       </c>
       <c r="Q126" s="42"/>
     </row>
-    <row r="127" spans="1:17">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A127" s="28">
         <v>69</v>
       </c>
@@ -11027,7 +11027,7 @@
       </c>
       <c r="Q127" s="42"/>
     </row>
-    <row r="128" spans="1:17">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A128" s="28"/>
       <c r="B128" s="21"/>
       <c r="C128" s="28">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="Q128" s="42"/>
     </row>
-    <row r="129" spans="1:17">
+    <row r="129" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A129" s="28"/>
       <c r="B129" s="21"/>
       <c r="C129" s="28">
@@ -11085,7 +11085,7 @@
       </c>
       <c r="Q129" s="42"/>
     </row>
-    <row r="130" spans="1:17">
+    <row r="130" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A130" s="28">
         <v>70</v>
       </c>
@@ -11100,7 +11100,7 @@
         <v>441</v>
       </c>
       <c r="F130" s="92" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="G130" s="28">
         <v>213</v>
@@ -11124,7 +11124,7 @@
       </c>
       <c r="Q130" s="35"/>
     </row>
-    <row r="131" spans="1:17">
+    <row r="131" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A131" s="28"/>
       <c r="B131" s="21"/>
       <c r="C131" s="28">
@@ -11135,7 +11135,7 @@
         <v>441</v>
       </c>
       <c r="F131" s="92" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="G131" s="28"/>
       <c r="H131" s="28"/>
@@ -11153,7 +11153,7 @@
       </c>
       <c r="Q131" s="35"/>
     </row>
-    <row r="132" spans="1:17">
+    <row r="132" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A132" s="28"/>
       <c r="B132" s="21"/>
       <c r="C132" s="28">
@@ -11164,7 +11164,7 @@
         <v>441</v>
       </c>
       <c r="F132" s="92" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="G132" s="28"/>
       <c r="H132" s="28"/>
@@ -11182,7 +11182,7 @@
       </c>
       <c r="Q132" s="35"/>
     </row>
-    <row r="133" spans="1:17">
+    <row r="133" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A133" s="36">
         <v>72</v>
       </c>
@@ -11212,7 +11212,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="134" spans="1:17">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A134" s="36">
         <v>73</v>
       </c>
@@ -11248,7 +11248,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="135" spans="1:17">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A135" s="36"/>
       <c r="B135" s="3"/>
       <c r="C135" s="36">
@@ -11276,7 +11276,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="136" spans="1:17">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A136" s="36">
         <v>75</v>
       </c>
@@ -11314,7 +11314,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="137" spans="1:17">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A137" s="36"/>
       <c r="B137" s="3"/>
       <c r="C137" s="36">
@@ -11342,7 +11342,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="138" spans="1:17">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A138" s="36"/>
       <c r="B138" s="3"/>
       <c r="C138" s="36">
@@ -11370,7 +11370,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="139" spans="1:17">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A139" s="36">
         <v>76</v>
       </c>
@@ -11410,7 +11410,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="140" spans="1:17">
+    <row r="140" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A140" s="36">
         <v>78</v>
       </c>
@@ -11449,7 +11449,7 @@
       </c>
       <c r="Q140" s="35"/>
     </row>
-    <row r="141" spans="1:17">
+    <row r="141" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A141" s="36"/>
       <c r="B141" s="3"/>
       <c r="C141" s="36">
@@ -11478,7 +11478,7 @@
       </c>
       <c r="Q141" s="35"/>
     </row>
-    <row r="142" spans="1:17">
+    <row r="142" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A142" s="36"/>
       <c r="B142" s="3"/>
       <c r="C142" s="36">
@@ -11507,7 +11507,7 @@
       </c>
       <c r="Q142" s="35"/>
     </row>
-    <row r="143" spans="1:17">
+    <row r="143" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A143" s="36">
         <v>79</v>
       </c>
@@ -11550,7 +11550,7 @@
       </c>
       <c r="Q143" s="42"/>
     </row>
-    <row r="144" spans="1:17">
+    <row r="144" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A144" s="28">
         <v>80</v>
       </c>
@@ -11583,7 +11583,7 @@
       </c>
       <c r="Q144" s="35"/>
     </row>
-    <row r="145" spans="1:17">
+    <row r="145" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A145" s="28">
         <v>81</v>
       </c>
@@ -11622,7 +11622,7 @@
       </c>
       <c r="Q145" s="35"/>
     </row>
-    <row r="146" spans="1:17">
+    <row r="146" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A146" s="28">
         <v>82</v>
       </c>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="Q146" s="35"/>
     </row>
-    <row r="147" spans="1:17">
+    <row r="147" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A147" s="28">
         <v>83</v>
       </c>
@@ -11704,7 +11704,7 @@
       </c>
       <c r="Q147" s="35"/>
     </row>
-    <row r="148" spans="1:17">
+    <row r="148" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A148" s="28"/>
       <c r="B148" s="21"/>
       <c r="C148" s="28">
@@ -11733,7 +11733,7 @@
       </c>
       <c r="Q148" s="35"/>
     </row>
-    <row r="149" spans="1:17">
+    <row r="149" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A149" s="28">
         <v>84</v>
       </c>
@@ -11774,7 +11774,7 @@
       </c>
       <c r="Q149" s="42"/>
     </row>
-    <row r="150" spans="1:17">
+    <row r="150" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A150" s="28"/>
       <c r="B150" s="21"/>
       <c r="C150" s="28">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="Q150" s="42"/>
     </row>
-    <row r="151" spans="1:17">
+    <row r="151" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A151" s="28"/>
       <c r="B151" s="21"/>
       <c r="C151" s="28">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="Q151" s="42"/>
     </row>
-    <row r="152" spans="1:17">
+    <row r="152" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A152" s="36">
         <v>206</v>
       </c>
@@ -11863,7 +11863,7 @@
       </c>
       <c r="Q152" s="35"/>
     </row>
-    <row r="153" spans="1:17">
+    <row r="153" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A153" s="36">
         <v>85</v>
       </c>
@@ -11873,7 +11873,7 @@
       </c>
       <c r="D153" s="3"/>
       <c r="E153" s="89" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F153" s="41" t="s">
         <v>164</v>
@@ -11902,7 +11902,7 @@
       </c>
       <c r="Q153" s="42"/>
     </row>
-    <row r="154" spans="1:17">
+    <row r="154" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A154" s="36"/>
       <c r="B154" s="3"/>
       <c r="C154" s="36">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="D154" s="3"/>
       <c r="E154" s="89" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F154" s="41" t="s">
         <v>164</v>
@@ -11931,7 +11931,7 @@
       </c>
       <c r="Q154" s="42"/>
     </row>
-    <row r="155" spans="1:17">
+    <row r="155" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A155" s="36"/>
       <c r="B155" s="3"/>
       <c r="C155" s="36">
@@ -11939,7 +11939,7 @@
       </c>
       <c r="D155" s="3"/>
       <c r="E155" s="89" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F155" s="41" t="s">
         <v>164</v>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="Q155" s="42"/>
     </row>
-    <row r="156" spans="1:17">
+    <row r="156" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A156" s="36"/>
       <c r="B156" s="3"/>
       <c r="C156" s="36">
@@ -11968,7 +11968,7 @@
       </c>
       <c r="D156" s="3"/>
       <c r="E156" s="89" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F156" s="41" t="s">
         <v>165</v>
@@ -11993,7 +11993,7 @@
       </c>
       <c r="Q156" s="35"/>
     </row>
-    <row r="157" spans="1:17">
+    <row r="157" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A157" s="36">
         <v>86</v>
       </c>
@@ -12005,7 +12005,7 @@
       </c>
       <c r="D157" s="3"/>
       <c r="E157" s="89" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F157" s="41" t="s">
         <v>155</v>
@@ -12034,7 +12034,7 @@
       </c>
       <c r="Q157" s="35"/>
     </row>
-    <row r="158" spans="1:17">
+    <row r="158" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A158" s="36"/>
       <c r="B158" s="3"/>
       <c r="C158" s="36">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="D158" s="3"/>
       <c r="E158" s="89" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F158" s="41" t="s">
         <v>155</v>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="Q158" s="35"/>
     </row>
-    <row r="159" spans="1:17">
+    <row r="159" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A159" s="36">
         <v>87</v>
       </c>
@@ -12075,7 +12075,7 @@
       </c>
       <c r="D159" s="3"/>
       <c r="E159" s="89" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F159" s="41" t="s">
         <v>153</v>
@@ -12104,7 +12104,7 @@
       </c>
       <c r="Q159" s="35"/>
     </row>
-    <row r="160" spans="1:17">
+    <row r="160" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A160" s="36">
         <v>88</v>
       </c>
@@ -12116,7 +12116,7 @@
       </c>
       <c r="D160" s="3"/>
       <c r="E160" s="89" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="F160" s="41" t="s">
         <v>166</v>
@@ -12145,7 +12145,7 @@
       </c>
       <c r="Q160" s="35"/>
     </row>
-    <row r="161" spans="1:17">
+    <row r="161" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A161" s="36">
         <v>89</v>
       </c>
@@ -12157,7 +12157,7 @@
       </c>
       <c r="D161" s="3"/>
       <c r="E161" s="89" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F161" s="41" t="s">
         <v>167</v>
@@ -12186,7 +12186,7 @@
       </c>
       <c r="Q161" s="35"/>
     </row>
-    <row r="162" spans="1:17">
+    <row r="162" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A162" s="36">
         <v>90</v>
       </c>
@@ -12198,7 +12198,7 @@
       </c>
       <c r="D162" s="3"/>
       <c r="E162" s="89" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="F162" s="41" t="s">
         <v>168</v>
@@ -12227,7 +12227,7 @@
       </c>
       <c r="Q162" s="35"/>
     </row>
-    <row r="163" spans="1:17">
+    <row r="163" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A163" s="36">
         <v>91</v>
       </c>
@@ -12239,7 +12239,7 @@
       </c>
       <c r="D163" s="3"/>
       <c r="E163" s="89" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="F163" s="49" t="s">
         <v>505</v>
@@ -12268,7 +12268,7 @@
       </c>
       <c r="Q163" s="35"/>
     </row>
-    <row r="164" spans="1:17">
+    <row r="164" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A164" s="36">
         <v>92</v>
       </c>
@@ -12280,7 +12280,7 @@
       </c>
       <c r="D164" s="3"/>
       <c r="E164" s="89" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="F164" s="41" t="s">
         <v>170</v>
@@ -12309,7 +12309,7 @@
       </c>
       <c r="Q164" s="42"/>
     </row>
-    <row r="165" spans="1:17">
+    <row r="165" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A165" s="28">
         <v>93</v>
       </c>
@@ -12344,7 +12344,7 @@
       </c>
       <c r="Q165" s="35"/>
     </row>
-    <row r="166" spans="1:17">
+    <row r="166" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A166" s="28"/>
       <c r="B166" s="21"/>
       <c r="C166" s="28">
@@ -12371,7 +12371,7 @@
       </c>
       <c r="Q166" s="35"/>
     </row>
-    <row r="167" spans="1:17">
+    <row r="167" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A167" s="28">
         <v>94</v>
       </c>
@@ -12410,7 +12410,7 @@
       </c>
       <c r="Q167" s="35"/>
     </row>
-    <row r="168" spans="1:17">
+    <row r="168" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A168" s="28">
         <v>95</v>
       </c>
@@ -12451,7 +12451,7 @@
       </c>
       <c r="Q168" s="35"/>
     </row>
-    <row r="169" spans="1:17">
+    <row r="169" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A169" s="28"/>
       <c r="B169" s="21"/>
       <c r="C169" s="28">
@@ -12478,7 +12478,7 @@
       <c r="P169" s="2"/>
       <c r="Q169" s="35"/>
     </row>
-    <row r="170" spans="1:17">
+    <row r="170" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A170" s="28"/>
       <c r="B170" s="21"/>
       <c r="C170" s="28">
@@ -12507,7 +12507,7 @@
       <c r="P170" s="2"/>
       <c r="Q170" s="35"/>
     </row>
-    <row r="171" spans="1:17">
+    <row r="171" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A171" s="28">
         <v>96</v>
       </c>
@@ -12550,7 +12550,7 @@
       </c>
       <c r="Q171" s="35"/>
     </row>
-    <row r="172" spans="1:17">
+    <row r="172" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A172" s="28">
         <v>97</v>
       </c>
@@ -12593,7 +12593,7 @@
       </c>
       <c r="Q172" s="35"/>
     </row>
-    <row r="173" spans="1:17">
+    <row r="173" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A173" s="28"/>
       <c r="B173" s="21"/>
       <c r="C173" s="28">
@@ -12622,7 +12622,7 @@
       <c r="P173" s="2"/>
       <c r="Q173" s="35"/>
     </row>
-    <row r="174" spans="1:17">
+    <row r="174" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A174" s="36">
         <v>207</v>
       </c>
@@ -12633,7 +12633,7 @@
       <c r="D174" s="3"/>
       <c r="E174" s="3"/>
       <c r="F174" s="89" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="G174" s="36">
         <v>43</v>
@@ -12653,7 +12653,7 @@
       </c>
       <c r="Q174" s="35"/>
     </row>
-    <row r="175" spans="1:17">
+    <row r="175" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A175" s="36">
         <v>98</v>
       </c>
@@ -12663,10 +12663,10 @@
       </c>
       <c r="D175" s="3"/>
       <c r="E175" s="89" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="F175" s="89" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="G175" s="36">
         <v>207</v>
@@ -12690,7 +12690,7 @@
       <c r="P175" s="1"/>
       <c r="Q175" s="35"/>
     </row>
-    <row r="176" spans="1:17">
+    <row r="176" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A176" s="36">
         <v>99</v>
       </c>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="D176" s="3"/>
       <c r="E176" s="89" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F176" s="41" t="s">
         <v>176</v>
@@ -12730,7 +12730,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="177" spans="1:17">
+    <row r="177" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A177" s="36"/>
       <c r="B177" s="3"/>
       <c r="C177" s="36">
@@ -12738,7 +12738,7 @@
       </c>
       <c r="D177" s="3"/>
       <c r="E177" s="89" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F177" s="41" t="s">
         <v>176</v>
@@ -12758,7 +12758,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="178" spans="1:17">
+    <row r="178" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A178" s="28">
         <v>100</v>
       </c>
@@ -12789,7 +12789,7 @@
       </c>
       <c r="Q178" s="35"/>
     </row>
-    <row r="179" spans="1:17">
+    <row r="179" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A179" s="28">
         <v>101</v>
       </c>
@@ -12828,7 +12828,7 @@
       </c>
       <c r="Q179" s="35"/>
     </row>
-    <row r="180" spans="1:17">
+    <row r="180" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A180" s="28"/>
       <c r="B180" s="21"/>
       <c r="C180" s="28">
@@ -12857,7 +12857,7 @@
       </c>
       <c r="Q180" s="35"/>
     </row>
-    <row r="181" spans="1:17">
+    <row r="181" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A181" s="28">
         <v>102</v>
       </c>
@@ -12869,7 +12869,7 @@
       </c>
       <c r="D181" s="21"/>
       <c r="E181" s="88" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="F181" s="33" t="s">
         <v>179</v>
@@ -12898,7 +12898,7 @@
       </c>
       <c r="Q181" s="35"/>
     </row>
-    <row r="182" spans="1:17">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A182" s="28"/>
       <c r="B182" s="21"/>
       <c r="C182" s="28">
@@ -12906,7 +12906,7 @@
       </c>
       <c r="D182" s="21"/>
       <c r="E182" s="88" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="F182" s="21"/>
       <c r="G182" s="28"/>
@@ -12929,7 +12929,7 @@
       </c>
       <c r="Q182" s="42"/>
     </row>
-    <row r="183" spans="1:17">
+    <row r="183" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A183" s="36">
         <v>103</v>
       </c>
@@ -12960,7 +12960,7 @@
       </c>
       <c r="Q183" s="35"/>
     </row>
-    <row r="184" spans="1:17">
+    <row r="184" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A184" s="28">
         <v>71</v>
       </c>
@@ -12998,7 +12998,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="185" spans="1:17">
+    <row r="185" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A185" s="36">
         <v>104</v>
       </c>
@@ -13039,7 +13039,7 @@
       </c>
       <c r="Q185" s="35"/>
     </row>
-    <row r="186" spans="1:17">
+    <row r="186" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A186" s="36">
         <v>105</v>
       </c>
@@ -13082,7 +13082,7 @@
       </c>
       <c r="Q186" s="35"/>
     </row>
-    <row r="187" spans="1:17">
+    <row r="187" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A187" s="36">
         <v>106</v>
       </c>
@@ -13124,7 +13124,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="188" spans="1:17">
+    <row r="188" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A188" s="28">
         <v>107</v>
       </c>
@@ -13162,7 +13162,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="189" spans="1:17">
+    <row r="189" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A189" s="28"/>
       <c r="B189" s="21"/>
       <c r="C189" s="28">
@@ -13190,7 +13190,7 @@
       <c r="O189" s="2"/>
       <c r="P189" s="2"/>
     </row>
-    <row r="190" spans="1:17">
+    <row r="190" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A190" s="28"/>
       <c r="B190" s="21"/>
       <c r="C190" s="28">
@@ -13218,7 +13218,7 @@
       <c r="O190" s="2"/>
       <c r="P190" s="2"/>
     </row>
-    <row r="191" spans="1:17">
+    <row r="191" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A191" s="36">
         <v>209</v>
       </c>
@@ -13248,7 +13248,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="192" spans="1:17">
+    <row r="192" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A192" s="36">
         <v>108</v>
       </c>
@@ -13258,7 +13258,7 @@
       </c>
       <c r="D192" s="3"/>
       <c r="E192" s="89" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F192" s="3" t="s">
         <v>184</v>
@@ -13282,7 +13282,7 @@
       <c r="O192" s="1"/>
       <c r="P192" s="1"/>
     </row>
-    <row r="193" spans="1:16">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A193" s="36">
         <v>109</v>
       </c>
@@ -13294,7 +13294,7 @@
       </c>
       <c r="D193" s="3"/>
       <c r="E193" s="89" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="F193" s="41" t="s">
         <v>185</v>
@@ -13320,11 +13320,11 @@
         <v>569</v>
       </c>
     </row>
-    <row r="194" spans="1:16">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A194" s="61"/>
       <c r="C194" s="61"/>
     </row>
-    <row r="195" spans="1:16">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A195" s="61"/>
       <c r="C195" s="61"/>
     </row>
@@ -13361,26 +13361,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="4" width="7.140625" customWidth="1"/>
+    <col min="1" max="2" width="35.6640625" customWidth="1"/>
+    <col min="3" max="4" width="7.1640625" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
-    <col min="6" max="8" width="28.42578125" customWidth="1"/>
-    <col min="10" max="10" width="42.85546875" customWidth="1"/>
+    <col min="6" max="8" width="28.5" customWidth="1"/>
+    <col min="10" max="10" width="42.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="96" t="s">
         <v>2</v>
       </c>
@@ -13405,7 +13405,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="45">
+    <row r="5" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="97"/>
       <c r="B5" s="97"/>
       <c r="C5" s="1" t="s">
@@ -13422,7 +13422,7 @@
       </c>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" ht="45">
+    <row r="6" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="21"/>
       <c r="B6" s="21"/>
       <c r="C6" s="2"/>
@@ -13441,7 +13441,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="60">
+    <row r="7" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A7" s="21"/>
       <c r="B7" s="21"/>
       <c r="C7" s="2"/>
@@ -13458,7 +13458,7 @@
       </c>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" ht="60">
+    <row r="8" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A8" s="21"/>
       <c r="B8" s="21"/>
       <c r="C8" s="2"/>
@@ -13475,7 +13475,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="30">
+    <row r="9" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="21"/>
       <c r="B9" s="21"/>
       <c r="C9" s="2"/>
@@ -13492,7 +13492,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="30">
+    <row r="10" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="21"/>
       <c r="B10" s="21"/>
       <c r="C10" s="2"/>
@@ -13511,7 +13511,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30">
+    <row r="11" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="21"/>
       <c r="B11" s="21"/>
       <c r="C11" s="2"/>
@@ -13530,7 +13530,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="30">
+    <row r="12" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="21"/>
       <c r="B12" s="21"/>
       <c r="C12" s="2"/>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10" ht="30">
+    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="21"/>
       <c r="B13" s="21"/>
       <c r="C13" s="2"/>
@@ -13564,7 +13564,7 @@
       </c>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10" ht="30">
+    <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="21"/>
       <c r="B14" s="21"/>
       <c r="C14" s="2"/>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" ht="30">
+    <row r="15" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="21"/>
       <c r="B15" s="21"/>
       <c r="C15" s="2"/>
@@ -13598,7 +13598,7 @@
       </c>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10" ht="60">
+    <row r="16" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A16" s="21"/>
       <c r="B16" s="21"/>
       <c r="C16" s="2"/>
@@ -13611,7 +13611,7 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="1:10" ht="75">
+    <row r="17" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A17" s="21"/>
       <c r="B17" s="21"/>
       <c r="C17" s="2"/>
@@ -13624,11 +13624,11 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="62"/>
       <c r="B18" s="62"/>
     </row>
-    <row r="19" spans="1:10" ht="45">
+    <row r="19" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>77</v>
       </c>

</xml_diff>